<commit_message>
fix unit tests for windio v2
</commit_message>
<xml_diff>
--- a/Documentation/IEA-15-240-RWT_tabular.xlsx
+++ b/Documentation/IEA-15-240-RWT_tabular.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gbarter/devel/IEA-15-240-RWT/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46DBE723-B685-144D-BC48-09682C209726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{126B7BE3-3AFE-C946-B584-E06D5408FAB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17020" yWindow="500" windowWidth="33600" windowHeight="19360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,20 @@
     <sheet name="Rotor Performance" sheetId="17" r:id="rId18"/>
     <sheet name="Nacelle Mass Properties" sheetId="18" r:id="rId19"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -996,7 +1009,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="2"/>
@@ -1004,6 +1017,7 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Heading 1" xfId="2" builtinId="16"/>
@@ -13234,7 +13248,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
-  <dimension ref="A1:K77"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
@@ -13388,7 +13402,7 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B5">
-        <v>-27.5</v>
+        <v>-25</v>
       </c>
       <c r="C5">
         <v>10</v>
@@ -13420,2314 +13434,1162 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B6">
-        <v>-27.498999999999999</v>
+        <v>-24.998999999999999</v>
       </c>
       <c r="C6">
         <v>10</v>
       </c>
       <c r="D6">
-        <v>55.341000000000001</v>
+        <v>53.448999999999998</v>
       </c>
       <c r="E6">
-        <v>14429.960803688969</v>
+        <v>13939.280294147429</v>
       </c>
       <c r="F6">
-        <v>178389.13728831729</v>
+        <v>172388.3576143948</v>
       </c>
       <c r="G6">
-        <v>178389.13728831729</v>
+        <v>172388.3576143948</v>
       </c>
       <c r="H6">
-        <v>4274841535785.2231</v>
+        <v>4131041399817.752</v>
       </c>
       <c r="I6">
-        <v>4274841535785.2231</v>
+        <v>4131041399817.752</v>
       </c>
       <c r="J6">
-        <v>3389949337877.6821</v>
+        <v>3275915830055.478</v>
       </c>
       <c r="K6">
-        <v>345793453239.61108</v>
+        <v>334034993868.85773</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B7">
-        <v>-25</v>
+        <v>-20</v>
       </c>
       <c r="C7">
         <v>10</v>
       </c>
       <c r="D7">
-        <v>55.341000000000001</v>
+        <v>53.448999999999998</v>
       </c>
       <c r="E7">
-        <v>14429.960803688969</v>
+        <v>13939.280294147429</v>
       </c>
       <c r="F7">
-        <v>178389.13728831729</v>
+        <v>172388.3576143948</v>
       </c>
       <c r="G7">
-        <v>178389.13728831729</v>
+        <v>172388.3576143948</v>
       </c>
       <c r="H7">
-        <v>4274841535785.2231</v>
+        <v>4131041399817.752</v>
       </c>
       <c r="I7">
-        <v>4274841535785.2231</v>
+        <v>4131041399817.752</v>
       </c>
       <c r="J7">
-        <v>3389949337877.6821</v>
+        <v>3275915830055.478</v>
       </c>
       <c r="K7">
-        <v>345793453239.61108</v>
+        <v>334034993868.85773</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B8">
-        <v>-24.998999999999999</v>
+        <v>-19.998999999999999</v>
       </c>
       <c r="C8">
         <v>10</v>
       </c>
       <c r="D8">
-        <v>54.395000000000003</v>
+        <v>51.509</v>
       </c>
       <c r="E8">
-        <v>14184.64401337621</v>
+        <v>13435.95631086556</v>
       </c>
       <c r="F8">
-        <v>175389.60832743839</v>
+        <v>166228.18419461499</v>
       </c>
       <c r="G8">
-        <v>175389.60832743839</v>
+        <v>166228.18419461499</v>
       </c>
       <c r="H8">
-        <v>4202962097470.3682</v>
+        <v>3983421619808.6509</v>
       </c>
       <c r="I8">
-        <v>4202962097470.3682</v>
+        <v>3983421619808.6509</v>
       </c>
       <c r="J8">
-        <v>3332948943294.001</v>
+        <v>3158853344508.2598</v>
       </c>
       <c r="K8">
-        <v>339914785846.54242</v>
+        <v>321973551662.24689</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B9">
-        <v>-24.998999999999999</v>
+        <v>-15</v>
       </c>
       <c r="C9">
         <v>10</v>
       </c>
       <c r="D9">
-        <v>54.395000000000003</v>
+        <v>51.509</v>
       </c>
       <c r="E9">
-        <v>14184.64401337621</v>
+        <v>13435.95631086556</v>
       </c>
       <c r="F9">
-        <v>175389.60832743839</v>
+        <v>166228.18419461499</v>
       </c>
       <c r="G9">
-        <v>175389.60832743839</v>
+        <v>166228.18419461499</v>
       </c>
       <c r="H9">
-        <v>4202962097470.3682</v>
+        <v>3983421619808.6509</v>
       </c>
       <c r="I9">
-        <v>4202962097470.3682</v>
+        <v>3983421619808.6509</v>
       </c>
       <c r="J9">
-        <v>3332948943294.001</v>
+        <v>3158853344508.2598</v>
       </c>
       <c r="K9">
-        <v>339914785846.54242</v>
+        <v>321973551662.24689</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B10">
-        <v>-24.998000000000001</v>
+        <v>-14.999000000000001</v>
       </c>
       <c r="C10">
         <v>10</v>
       </c>
       <c r="D10">
-        <v>53.448999999999998</v>
+        <v>49.527000000000001</v>
       </c>
       <c r="E10">
-        <v>13939.280294147429</v>
+        <v>12921.531806218951</v>
       </c>
       <c r="F10">
-        <v>172388.3576143948</v>
+        <v>159927.1596963164</v>
       </c>
       <c r="G10">
-        <v>172388.3576143948</v>
+        <v>159927.1596963164</v>
       </c>
       <c r="H10">
-        <v>4131041399817.752</v>
+        <v>3832426544364.1611</v>
       </c>
       <c r="I10">
-        <v>4131041399817.752</v>
+        <v>3832426544364.1611</v>
       </c>
       <c r="J10">
-        <v>3275915830055.478</v>
+        <v>3039114249680.7788</v>
       </c>
       <c r="K10">
-        <v>334034993868.85773</v>
+        <v>309646101275.31641</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B11">
-        <v>-20</v>
+        <v>-10</v>
       </c>
       <c r="C11">
         <v>10</v>
       </c>
       <c r="D11">
-        <v>53.448999999999998</v>
+        <v>49.527000000000001</v>
       </c>
       <c r="E11">
-        <v>13939.280294147429</v>
+        <v>12921.531806218951</v>
       </c>
       <c r="F11">
-        <v>172388.3576143948</v>
+        <v>159927.1596963164</v>
       </c>
       <c r="G11">
-        <v>172388.3576143948</v>
+        <v>159927.1596963164</v>
       </c>
       <c r="H11">
-        <v>4131041399817.752</v>
+        <v>3832426544364.1611</v>
       </c>
       <c r="I11">
-        <v>4131041399817.752</v>
+        <v>3832426544364.1611</v>
       </c>
       <c r="J11">
-        <v>3275915830055.478</v>
+        <v>3039114249680.7788</v>
       </c>
       <c r="K11">
-        <v>334034993868.85773</v>
+        <v>309646101275.31641</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B12">
-        <v>-19.998999999999999</v>
+        <v>-9.9990000000000006</v>
       </c>
       <c r="C12">
         <v>10</v>
       </c>
       <c r="D12">
-        <v>52.478999999999999</v>
+        <v>47.517000000000003</v>
       </c>
       <c r="E12">
-        <v>13687.642972652549</v>
+        <v>12399.629567330059</v>
       </c>
       <c r="F12">
-        <v>169309.17671693451</v>
+        <v>153529.38576954859</v>
       </c>
       <c r="G12">
-        <v>169309.17671693451</v>
+        <v>153529.38576954859</v>
       </c>
       <c r="H12">
-        <v>4057253216317.624</v>
+        <v>3679113006698.9839</v>
       </c>
       <c r="I12">
-        <v>4057253216317.624</v>
+        <v>3679113006698.9839</v>
       </c>
       <c r="J12">
-        <v>3217401800539.876</v>
+        <v>2917536614312.2939</v>
       </c>
       <c r="K12">
-        <v>328004863950.45648</v>
+        <v>297139457640.30811</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B13">
-        <v>-19.998999999999999</v>
+        <v>-5</v>
       </c>
       <c r="C13">
         <v>10</v>
       </c>
       <c r="D13">
-        <v>52.478999999999999</v>
+        <v>47.517000000000003</v>
       </c>
       <c r="E13">
-        <v>13687.642972652549</v>
+        <v>12399.629567330059</v>
       </c>
       <c r="F13">
-        <v>169309.17671693451</v>
+        <v>153529.38576954859</v>
       </c>
       <c r="G13">
-        <v>169309.17671693451</v>
+        <v>153529.38576954859</v>
       </c>
       <c r="H13">
-        <v>4057253216317.624</v>
+        <v>3679113006698.9839</v>
       </c>
       <c r="I13">
-        <v>4057253216317.624</v>
+        <v>3679113006698.9839</v>
       </c>
       <c r="J13">
-        <v>3217401800539.876</v>
+        <v>2917536614312.2939</v>
       </c>
       <c r="K13">
-        <v>328004863950.45648</v>
+        <v>297139457640.30811</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B14">
-        <v>-19.998000000000001</v>
+        <v>-4.9989999999999997</v>
       </c>
       <c r="C14">
         <v>10</v>
       </c>
       <c r="D14">
-        <v>51.509</v>
+        <v>45.517000000000003</v>
       </c>
       <c r="E14">
-        <v>13435.95631086556</v>
+        <v>11880.11357474014</v>
       </c>
       <c r="F14">
-        <v>166228.18419461499</v>
+        <v>147155.7051570719</v>
       </c>
       <c r="G14">
-        <v>166228.18419461499</v>
+        <v>147155.7051570719</v>
       </c>
       <c r="H14">
-        <v>3983421619808.6509</v>
+        <v>3526376830986.626</v>
       </c>
       <c r="I14">
-        <v>3983421619808.6509</v>
+        <v>3526376830986.626</v>
       </c>
       <c r="J14">
-        <v>3158853344508.2598</v>
+        <v>2796416826972.395</v>
       </c>
       <c r="K14">
-        <v>321973551662.24689</v>
+        <v>284689996998.32593</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>193</v>
+      </c>
       <c r="B15">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="C15">
         <v>10</v>
       </c>
       <c r="D15">
-        <v>51.509</v>
+        <v>45.517000000000003</v>
       </c>
       <c r="E15">
-        <v>13435.95631086556</v>
+        <v>11880.11357474014</v>
       </c>
       <c r="F15">
-        <v>166228.18419461499</v>
+        <v>147155.7051570719</v>
       </c>
       <c r="G15">
-        <v>166228.18419461499</v>
+        <v>147155.7051570719</v>
       </c>
       <c r="H15">
-        <v>3983421619808.6509</v>
+        <v>3526376830986.626</v>
       </c>
       <c r="I15">
-        <v>3983421619808.6509</v>
+        <v>3526376830986.626</v>
       </c>
       <c r="J15">
-        <v>3158853344508.2598</v>
+        <v>2796416826972.395</v>
       </c>
       <c r="K15">
-        <v>321973551662.24689</v>
+        <v>284689996998.32593</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B16">
-        <v>-14.999000000000001</v>
+        <v>1E-3</v>
       </c>
       <c r="C16">
         <v>10</v>
       </c>
       <c r="D16">
-        <v>50.518000000000001</v>
+        <v>43.527000000000001</v>
       </c>
       <c r="E16">
-        <v>13178.76980844315</v>
+        <v>11362.9869748166</v>
       </c>
       <c r="F16">
-        <v>163078.61815282659</v>
+        <v>140806.22742808619</v>
       </c>
       <c r="G16">
-        <v>163078.61815282659</v>
+        <v>140806.22742808619</v>
       </c>
       <c r="H16">
-        <v>3907946756597.8101</v>
+        <v>3374220642896.8662</v>
       </c>
       <c r="I16">
-        <v>3907946756597.8101</v>
+        <v>3374220642896.8662</v>
       </c>
       <c r="J16">
-        <v>3099001777982.063</v>
+        <v>2675756969817.2139</v>
       </c>
       <c r="K16">
-        <v>315810443528.47241</v>
+        <v>272297794747.58209</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B17">
-        <v>-14.999000000000001</v>
+        <v>5</v>
       </c>
       <c r="C17">
         <v>10</v>
       </c>
       <c r="D17">
-        <v>50.518000000000001</v>
+        <v>43.527000000000001</v>
       </c>
       <c r="E17">
-        <v>13178.76980844315</v>
+        <v>11362.9869748166</v>
       </c>
       <c r="F17">
-        <v>163078.61815282659</v>
+        <v>140806.22742808619</v>
       </c>
       <c r="G17">
-        <v>163078.61815282659</v>
+        <v>140806.22742808619</v>
       </c>
       <c r="H17">
-        <v>3907946756597.8101</v>
+        <v>3374220642896.8662</v>
       </c>
       <c r="I17">
-        <v>3907946756597.8101</v>
+        <v>3374220642896.8662</v>
       </c>
       <c r="J17">
-        <v>3099001777982.063</v>
+        <v>2675756969817.2139</v>
       </c>
       <c r="K17">
-        <v>315810443528.47241</v>
+        <v>272297794747.58209</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B18">
-        <v>-14.997999999999999</v>
+        <v>5.0010000000000003</v>
       </c>
       <c r="C18">
         <v>10</v>
       </c>
       <c r="D18">
-        <v>49.527000000000001</v>
+        <v>42.241999999999997</v>
       </c>
       <c r="E18">
-        <v>12921.531806218951</v>
+        <v>11028.95317461117</v>
       </c>
       <c r="F18">
-        <v>159927.1596963164</v>
+        <v>136702.1220616003</v>
       </c>
       <c r="G18">
-        <v>159927.1596963164</v>
+        <v>136702.1220616003</v>
       </c>
       <c r="H18">
-        <v>3832426544364.1611</v>
+        <v>3275871604639.355</v>
       </c>
       <c r="I18">
-        <v>3832426544364.1611</v>
+        <v>3275871604639.355</v>
       </c>
       <c r="J18">
-        <v>3039114249680.7788</v>
+        <v>2597766182479.0088</v>
       </c>
       <c r="K18">
-        <v>309646101275.31641</v>
+        <v>264293150601.75339</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B19">
-        <v>-10</v>
+        <v>10</v>
       </c>
       <c r="C19">
         <v>10</v>
       </c>
       <c r="D19">
-        <v>49.527000000000001</v>
+        <v>42.241999999999997</v>
       </c>
       <c r="E19">
-        <v>12921.531806218951</v>
+        <v>11028.95317461117</v>
       </c>
       <c r="F19">
-        <v>159927.1596963164</v>
+        <v>136702.1220616003</v>
       </c>
       <c r="G19">
-        <v>159927.1596963164</v>
+        <v>136702.1220616003</v>
       </c>
       <c r="H19">
-        <v>3832426544364.1611</v>
+        <v>3275871604639.355</v>
       </c>
       <c r="I19">
-        <v>3832426544364.1611</v>
+        <v>3275871604639.355</v>
       </c>
       <c r="J19">
-        <v>3039114249680.7788</v>
+        <v>2597766182479.0088</v>
       </c>
       <c r="K19">
-        <v>309646101275.31641</v>
+        <v>264293150601.75339</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B20">
-        <v>-9.9990000000000006</v>
+        <v>10.000999999999999</v>
       </c>
       <c r="C20">
         <v>10</v>
       </c>
       <c r="D20">
-        <v>48.521999999999998</v>
+        <v>41.058</v>
       </c>
       <c r="E20">
-        <v>12660.60716935962</v>
+        <v>10721.09752311486</v>
       </c>
       <c r="F20">
-        <v>156729.2466485856</v>
+        <v>132917.77028131139</v>
       </c>
       <c r="G20">
-        <v>156729.2466485856</v>
+        <v>132917.77028131139</v>
       </c>
       <c r="H20">
-        <v>3755793114032.7241</v>
+        <v>3185185005543.0488</v>
       </c>
       <c r="I20">
-        <v>3755793114032.7241</v>
+        <v>3185185005543.0488</v>
       </c>
       <c r="J20">
-        <v>2978343939427.9502</v>
+        <v>2525851709395.6382</v>
       </c>
       <c r="K20">
-        <v>303393414075.23657</v>
+        <v>256915828495.4436</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>194</v>
+      </c>
       <c r="B21">
-        <v>-9.9990000000000006</v>
+        <v>15</v>
       </c>
       <c r="C21">
         <v>10</v>
       </c>
       <c r="D21">
-        <v>48.521999999999998</v>
+        <v>41.058</v>
       </c>
       <c r="E21">
-        <v>12660.60716935962</v>
+        <v>10721.09752311486</v>
       </c>
       <c r="F21">
-        <v>156729.2466485856</v>
+        <v>132917.77028131139</v>
       </c>
       <c r="G21">
-        <v>156729.2466485856</v>
+        <v>132917.77028131139</v>
       </c>
       <c r="H21">
-        <v>3755793114032.7241</v>
+        <v>3185185005543.0488</v>
       </c>
       <c r="I21">
-        <v>3755793114032.7241</v>
+        <v>3185185005543.0488</v>
       </c>
       <c r="J21">
-        <v>2978343939427.9502</v>
+        <v>2525851709395.6382</v>
       </c>
       <c r="K21">
-        <v>303393414075.23657</v>
+        <v>256915828495.4436</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B22">
-        <v>-9.9979999999999993</v>
+        <v>15.000999999999999</v>
       </c>
       <c r="C22">
         <v>10</v>
       </c>
       <c r="D22">
-        <v>47.517000000000003</v>
+        <v>39.496000000000002</v>
       </c>
       <c r="E22">
-        <v>12399.629567330059</v>
+        <v>10314.844411733609</v>
       </c>
       <c r="F22">
-        <v>153529.38576954859</v>
+        <v>127921.09002862249</v>
       </c>
       <c r="G22">
-        <v>153529.38576954859</v>
+        <v>127921.09002862249</v>
       </c>
       <c r="H22">
-        <v>3679113006698.9839</v>
+        <v>3065446681730.708</v>
       </c>
       <c r="I22">
-        <v>3679113006698.9839</v>
+        <v>3065446681730.708</v>
       </c>
       <c r="J22">
-        <v>2917536614312.2939</v>
+        <v>2430899218612.4521</v>
       </c>
       <c r="K22">
-        <v>297139457640.30811</v>
+        <v>247180551443.41281</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B23">
-        <v>-5</v>
+        <v>28</v>
       </c>
       <c r="C23">
         <v>10</v>
       </c>
       <c r="D23">
-        <v>47.517000000000003</v>
+        <v>39.496000000000002</v>
       </c>
       <c r="E23">
-        <v>12399.629567330059</v>
+        <v>10314.844411733609</v>
       </c>
       <c r="F23">
-        <v>153529.38576954859</v>
+        <v>127921.09002862249</v>
       </c>
       <c r="G23">
-        <v>153529.38576954859</v>
+        <v>127921.09002862249</v>
       </c>
       <c r="H23">
-        <v>3679113006698.9839</v>
+        <v>3065446681730.708</v>
       </c>
       <c r="I23">
-        <v>3679113006698.9839</v>
+        <v>3065446681730.708</v>
       </c>
       <c r="J23">
-        <v>2917536614312.2939</v>
+        <v>2430899218612.4521</v>
       </c>
       <c r="K23">
-        <v>297139457640.30811</v>
+        <v>247180551443.41281</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B24">
-        <v>-4.9989999999999997</v>
+        <v>28.001000000000001</v>
       </c>
       <c r="C24">
         <v>10</v>
       </c>
       <c r="D24">
-        <v>46.517000000000003</v>
+        <v>36.456000000000003</v>
       </c>
       <c r="E24">
-        <v>12139.897790767271</v>
+        <v>9523.8185311774014</v>
       </c>
       <c r="F24">
-        <v>150343.51049342929</v>
+        <v>118182.8952025789</v>
       </c>
       <c r="G24">
-        <v>150343.51049342929</v>
+        <v>118182.8952025789</v>
       </c>
       <c r="H24">
-        <v>3602768044414.792</v>
+        <v>2832084716093.4321</v>
       </c>
       <c r="I24">
-        <v>3602768044414.792</v>
+        <v>2832084716093.4321</v>
       </c>
       <c r="J24">
-        <v>2856995059220.9312</v>
+        <v>2245843179862.0918</v>
       </c>
       <c r="K24">
-        <v>290915355637.84497</v>
+        <v>228224743138.6868</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B25">
-        <v>-4.9989999999999997</v>
+        <v>41</v>
       </c>
       <c r="C25">
-        <v>10</v>
+        <v>9.9260000000000002</v>
       </c>
       <c r="D25">
-        <v>46.517000000000003</v>
+        <v>36.456000000000003</v>
       </c>
       <c r="E25">
-        <v>12139.897790767271</v>
+        <v>9453.0844057189461</v>
       </c>
       <c r="F25">
-        <v>150343.51049342929</v>
+        <v>115569.1673620746</v>
       </c>
       <c r="G25">
-        <v>150343.51049342929</v>
+        <v>115569.1673620746</v>
       </c>
       <c r="H25">
-        <v>3602768044414.792</v>
+        <v>2769450452002.7461</v>
       </c>
       <c r="I25">
-        <v>3602768044414.792</v>
+        <v>2769450452002.7461</v>
       </c>
       <c r="J25">
-        <v>2856995059220.9312</v>
+        <v>2196174208438.178</v>
       </c>
       <c r="K25">
-        <v>290915355637.84497</v>
+        <v>226529700592.35431</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B26">
-        <v>-4.9980000000000002</v>
+        <v>41.000999999999998</v>
       </c>
       <c r="C26">
-        <v>10</v>
+        <v>9.9260000000000002</v>
       </c>
       <c r="D26">
-        <v>45.517000000000003</v>
+        <v>33.779000000000003</v>
       </c>
       <c r="E26">
-        <v>11880.11357474014</v>
+        <v>8761.3060592618385</v>
       </c>
       <c r="F26">
-        <v>147155.7051570719</v>
+        <v>107169.58508948211</v>
       </c>
       <c r="G26">
-        <v>147155.7051570719</v>
+        <v>107169.58508948211</v>
       </c>
       <c r="H26">
-        <v>3526376830986.626</v>
+        <v>2568166429175.2251</v>
       </c>
       <c r="I26">
-        <v>3526376830986.626</v>
+        <v>2568166429175.2251</v>
       </c>
       <c r="J26">
-        <v>2796416826972.395</v>
+        <v>2036555978335.9529</v>
       </c>
       <c r="K26">
-        <v>284689996998.32593</v>
+        <v>209952218050.84689</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>193</v>
-      </c>
       <c r="B27">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="C27">
-        <v>10</v>
+        <v>9.4429999999999996</v>
       </c>
       <c r="D27">
-        <v>45.517000000000003</v>
+        <v>33.779000000000003</v>
       </c>
       <c r="E27">
-        <v>11880.11357474014</v>
+        <v>8333.5243885306409</v>
       </c>
       <c r="F27">
-        <v>147155.7051570719</v>
+        <v>92225.636090311411</v>
       </c>
       <c r="G27">
-        <v>147155.7051570719</v>
+        <v>92225.636090311411</v>
       </c>
       <c r="H27">
-        <v>3526376830986.626</v>
+        <v>2210055981076.2378</v>
       </c>
       <c r="I27">
-        <v>3526376830986.626</v>
+        <v>2210055981076.2378</v>
       </c>
       <c r="J27">
-        <v>2796416826972.395</v>
+        <v>1752574392993.457</v>
       </c>
       <c r="K27">
-        <v>284689996998.32593</v>
+        <v>199701039744.32401</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B28">
-        <v>1E-3</v>
+        <v>54.000999999999998</v>
       </c>
       <c r="C28">
-        <v>10</v>
+        <v>9.4429999999999996</v>
       </c>
       <c r="D28">
-        <v>44.521999999999998</v>
+        <v>32.192</v>
       </c>
       <c r="E28">
-        <v>11621.5762329687</v>
+        <v>7943.339505959193</v>
       </c>
       <c r="F28">
-        <v>143981.92246624999</v>
+        <v>87937.081105321893</v>
       </c>
       <c r="G28">
-        <v>143981.92246624999</v>
+        <v>87937.081105321893</v>
       </c>
       <c r="H28">
-        <v>3450321650281.5718</v>
+        <v>2107286870484.5891</v>
       </c>
       <c r="I28">
-        <v>3450321650281.5718</v>
+        <v>2107286870484.5891</v>
       </c>
       <c r="J28">
-        <v>2736105068673.2871</v>
+        <v>1671078488294.2791</v>
       </c>
       <c r="K28">
-        <v>278494517924.00439</v>
+        <v>190350814904.366</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B29">
-        <v>1E-3</v>
+        <v>67</v>
       </c>
       <c r="C29">
-        <v>10</v>
+        <v>8.8330000000000002</v>
       </c>
       <c r="D29">
-        <v>44.521999999999998</v>
+        <v>32.192</v>
       </c>
       <c r="E29">
-        <v>11621.5762329687</v>
+        <v>7428.4594766741811</v>
       </c>
       <c r="F29">
-        <v>143981.92246624999</v>
+        <v>71921.655457150788</v>
       </c>
       <c r="G29">
-        <v>143981.92246624999</v>
+        <v>71921.655457150788</v>
       </c>
       <c r="H29">
-        <v>3450321650281.5718</v>
+        <v>1723500010954.967</v>
       </c>
       <c r="I29">
-        <v>3450321650281.5718</v>
+        <v>1723500010954.967</v>
       </c>
       <c r="J29">
-        <v>2736105068673.2871</v>
+        <v>1366735508687.2891</v>
       </c>
       <c r="K29">
-        <v>278494517924.00439</v>
+        <v>178012448518.43231</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B30">
-        <v>2E-3</v>
+        <v>67.001000000000005</v>
       </c>
       <c r="C30">
-        <v>10</v>
+        <v>8.8330000000000002</v>
       </c>
       <c r="D30">
-        <v>43.527000000000001</v>
+        <v>30.707999999999998</v>
       </c>
       <c r="E30">
-        <v>11362.9869748166</v>
+        <v>7087.214160266677</v>
       </c>
       <c r="F30">
-        <v>140806.22742808619</v>
+        <v>68640.809682709922</v>
       </c>
       <c r="G30">
-        <v>140806.22742808619</v>
+        <v>68640.809682709922</v>
       </c>
       <c r="H30">
-        <v>3374220642896.8662</v>
+        <v>1644879215976.7529</v>
       </c>
       <c r="I30">
-        <v>3374220642896.8662</v>
+        <v>1644879215976.7529</v>
       </c>
       <c r="J30">
-        <v>2675756969817.2139</v>
+        <v>1304389218269.5649</v>
       </c>
       <c r="K30">
-        <v>272297794747.58209</v>
+        <v>169834990660.59619</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B31">
-        <v>5</v>
+        <v>80</v>
       </c>
       <c r="C31">
-        <v>10</v>
+        <v>8.1509999999999998</v>
       </c>
       <c r="D31">
-        <v>43.527000000000001</v>
+        <v>30.707999999999998</v>
       </c>
       <c r="E31">
-        <v>11362.9869748166</v>
+        <v>6538.0980826244668</v>
       </c>
       <c r="F31">
-        <v>140806.22742808619</v>
+        <v>53890.34303307574</v>
       </c>
       <c r="G31">
-        <v>140806.22742808619</v>
+        <v>53890.34303307574</v>
       </c>
       <c r="H31">
-        <v>3374220642896.8662</v>
+        <v>1291405296742.769</v>
       </c>
       <c r="I31">
-        <v>3374220642896.8662</v>
+        <v>1291405296742.769</v>
       </c>
       <c r="J31">
-        <v>2675756969817.2139</v>
+        <v>1024084400317.016</v>
       </c>
       <c r="K31">
-        <v>272297794747.58209</v>
+        <v>156676206149.63971</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B32">
-        <v>5.0010000000000003</v>
+        <v>80.001000000000005</v>
       </c>
       <c r="C32">
-        <v>10</v>
+        <v>8.1509999999999998</v>
       </c>
       <c r="D32">
-        <v>42.884</v>
+        <v>29.100999999999999</v>
       </c>
       <c r="E32">
-        <v>11195.85092413538</v>
+        <v>6197.1748615481274</v>
       </c>
       <c r="F32">
-        <v>138752.97677141579</v>
+        <v>51100.424514406717</v>
       </c>
       <c r="G32">
-        <v>138752.97677141579</v>
+        <v>51100.424514406717</v>
       </c>
       <c r="H32">
-        <v>3325017416041.5952</v>
+        <v>1224548874057.1941</v>
       </c>
       <c r="I32">
-        <v>3325017416041.5952</v>
+        <v>1224548874057.1941</v>
       </c>
       <c r="J32">
-        <v>2636738810920.9849</v>
+        <v>971067257127.3551</v>
       </c>
       <c r="K32">
-        <v>268292617400.79999</v>
+        <v>148506466847.54681</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B33">
-        <v>5.0010000000000003</v>
+        <v>93</v>
       </c>
       <c r="C33">
-        <v>10</v>
+        <v>7.39</v>
       </c>
       <c r="D33">
-        <v>42.884</v>
+        <v>29.100999999999999</v>
       </c>
       <c r="E33">
-        <v>11195.85092413538</v>
+        <v>5616.5163148661431</v>
       </c>
       <c r="F33">
-        <v>138752.97677141579</v>
+        <v>38040.441011391602</v>
       </c>
       <c r="G33">
-        <v>138752.97677141579</v>
+        <v>38040.441011391602</v>
       </c>
       <c r="H33">
-        <v>3325017416041.5952</v>
+        <v>911584975111.22949</v>
       </c>
       <c r="I33">
-        <v>3325017416041.5952</v>
+        <v>911584975111.22949</v>
       </c>
       <c r="J33">
-        <v>2636738810920.9849</v>
+        <v>722886885263.20496</v>
       </c>
       <c r="K33">
-        <v>268292617400.79999</v>
+        <v>134591812002.54359</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B34">
-        <v>5.0019999999999998</v>
+        <v>93.001000000000005</v>
       </c>
       <c r="C34">
-        <v>10</v>
+        <v>7.39</v>
       </c>
       <c r="D34">
-        <v>42.241999999999997</v>
+        <v>27.213000000000001</v>
       </c>
       <c r="E34">
-        <v>11028.95317461117</v>
+        <v>5253.4779234371445</v>
       </c>
       <c r="F34">
-        <v>136702.1220616003</v>
+        <v>35599.7813771168</v>
       </c>
       <c r="G34">
-        <v>136702.1220616003</v>
+        <v>35599.7813771168</v>
       </c>
       <c r="H34">
-        <v>3275871604639.355</v>
+        <v>853098044023.88684</v>
       </c>
       <c r="I34">
-        <v>3275871604639.355</v>
+        <v>853098044023.88684</v>
       </c>
       <c r="J34">
-        <v>2597766182479.0088</v>
+        <v>676506748910.94226</v>
       </c>
       <c r="K34">
-        <v>264293150601.75339</v>
+        <v>125892114148.985</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B35">
-        <v>10</v>
+        <v>106</v>
       </c>
       <c r="C35">
-        <v>10</v>
+        <v>6.9089999999999998</v>
       </c>
       <c r="D35">
-        <v>42.241999999999997</v>
+        <v>27.213000000000001</v>
       </c>
       <c r="E35">
-        <v>11028.95317461117</v>
+        <v>4910.275969995676</v>
       </c>
       <c r="F35">
-        <v>136702.1220616003</v>
+        <v>29068.669776437349</v>
       </c>
       <c r="G35">
-        <v>136702.1220616003</v>
+        <v>29068.669776437349</v>
       </c>
       <c r="H35">
-        <v>3275871604639.355</v>
+        <v>696589258960.87573</v>
       </c>
       <c r="I35">
-        <v>3275871604639.355</v>
+        <v>696589258960.87573</v>
       </c>
       <c r="J35">
-        <v>2597766182479.0088</v>
+        <v>552395282355.97449</v>
       </c>
       <c r="K35">
-        <v>264293150601.75339</v>
+        <v>117667768272.1226</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B36">
-        <v>10.000999999999999</v>
+        <v>106.001</v>
       </c>
       <c r="C36">
-        <v>10</v>
+        <v>6.9089999999999998</v>
       </c>
       <c r="D36">
-        <v>41.65</v>
+        <v>24.009</v>
       </c>
       <c r="E36">
-        <v>10875.03453793534</v>
+        <v>4334.1676032059768</v>
       </c>
       <c r="F36">
-        <v>134810.28504470401</v>
+        <v>25681.93541283693</v>
       </c>
       <c r="G36">
-        <v>134810.28504470401</v>
+        <v>25681.93541283693</v>
       </c>
       <c r="H36">
-        <v>3230536425705.8242</v>
+        <v>615430994795.99658</v>
       </c>
       <c r="I36">
-        <v>3230536425705.8242</v>
+        <v>615430994795.99658</v>
       </c>
       <c r="J36">
-        <v>2561815385584.7192</v>
+        <v>488036778873.22522</v>
       </c>
       <c r="K36">
-        <v>260604709751.62579</v>
+        <v>103862152005.8945</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B37">
-        <v>10.000999999999999</v>
+        <v>119</v>
       </c>
       <c r="C37">
-        <v>10</v>
+        <v>6.7480000000000002</v>
       </c>
       <c r="D37">
-        <v>41.65</v>
+        <v>24.009</v>
       </c>
       <c r="E37">
-        <v>10875.03453793534</v>
+        <v>4232.8165652574853</v>
       </c>
       <c r="F37">
-        <v>134810.28504470401</v>
+        <v>23922.096893685812</v>
       </c>
       <c r="G37">
-        <v>134810.28504470401</v>
+        <v>23922.096893685812</v>
       </c>
       <c r="H37">
-        <v>3230536425705.8242</v>
+        <v>573258971811.30627</v>
       </c>
       <c r="I37">
-        <v>3230536425705.8242</v>
+        <v>573258971811.30627</v>
       </c>
       <c r="J37">
-        <v>2561815385584.7192</v>
+        <v>454594364646.36578</v>
       </c>
       <c r="K37">
-        <v>260604709751.62579</v>
+        <v>101433418769.6498</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B38">
-        <v>10.002000000000001</v>
+        <v>119.001</v>
       </c>
       <c r="C38">
-        <v>10</v>
+        <v>6.7480000000000002</v>
       </c>
       <c r="D38">
-        <v>41.058</v>
+        <v>20.826000000000001</v>
       </c>
       <c r="E38">
-        <v>10721.09752311486</v>
+        <v>3673.3877898387768</v>
       </c>
       <c r="F38">
-        <v>132917.77028131139</v>
+        <v>20780.03502692196</v>
       </c>
       <c r="G38">
-        <v>132917.77028131139</v>
+        <v>20780.03502692196</v>
       </c>
       <c r="H38">
-        <v>3185185005543.0488</v>
+        <v>497963935464.22137</v>
       </c>
       <c r="I38">
-        <v>3185185005543.0488</v>
+        <v>497963935464.22137</v>
       </c>
       <c r="J38">
-        <v>2525851709395.6382</v>
+        <v>394885400823.12762</v>
       </c>
       <c r="K38">
-        <v>256915828495.4436</v>
+        <v>88027505148.305237</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
-        <v>194</v>
-      </c>
       <c r="B39">
-        <v>15</v>
+        <v>132</v>
       </c>
       <c r="C39">
-        <v>10</v>
+        <v>6.5720000000000001</v>
       </c>
       <c r="D39">
-        <v>41.058</v>
+        <v>20.826000000000001</v>
       </c>
       <c r="E39">
-        <v>10721.09752311486</v>
+        <v>3577.282612388075</v>
       </c>
       <c r="F39">
-        <v>132917.77028131139</v>
+        <v>19191.367526978469</v>
       </c>
       <c r="G39">
-        <v>132917.77028131139</v>
+        <v>19191.367526978469</v>
       </c>
       <c r="H39">
-        <v>3185185005543.0488</v>
+        <v>459893782098.69342</v>
       </c>
       <c r="I39">
-        <v>3185185005543.0488</v>
+        <v>459893782098.69342</v>
       </c>
       <c r="J39">
-        <v>2525851709395.6382</v>
+        <v>364695769204.26392</v>
       </c>
       <c r="K39">
-        <v>256915828495.4436</v>
+        <v>85724481485.455917</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B40">
-        <v>15.000999999999999</v>
+        <v>132.001</v>
       </c>
       <c r="C40">
-        <v>10</v>
+        <v>6.5720000000000001</v>
       </c>
       <c r="D40">
-        <v>39.496000000000002</v>
+        <v>23.998000000000001</v>
       </c>
       <c r="E40">
-        <v>10314.844411733609</v>
+        <v>4120.1412531729766</v>
       </c>
       <c r="F40">
-        <v>127921.09002862249</v>
+        <v>22082.363701823171</v>
       </c>
       <c r="G40">
-        <v>127921.09002862249</v>
+        <v>22082.363701823171</v>
       </c>
       <c r="H40">
-        <v>3065446681730.708</v>
+        <v>529172386815.79602</v>
       </c>
       <c r="I40">
-        <v>3065446681730.708</v>
+        <v>529172386815.79602</v>
       </c>
       <c r="J40">
-        <v>2430899218612.4521</v>
+        <v>419633702744.92621</v>
       </c>
       <c r="K40">
-        <v>247180551443.41281</v>
+        <v>98733315436.687683</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>195</v>
+      </c>
       <c r="B41">
-        <v>28</v>
+        <v>144.386</v>
       </c>
       <c r="C41">
-        <v>10</v>
+        <v>6.5</v>
       </c>
       <c r="D41">
-        <v>39.496000000000002</v>
+        <v>23.998000000000001</v>
       </c>
       <c r="E41">
-        <v>10314.844411733609</v>
+        <v>4074.8373314227201</v>
       </c>
       <c r="F41">
-        <v>127921.09002862249</v>
+        <v>21361.915922655739</v>
       </c>
       <c r="G41">
-        <v>127921.09002862249</v>
+        <v>21361.915922655739</v>
       </c>
       <c r="H41">
-        <v>3065446681730.708</v>
+        <v>511907882162.8501</v>
       </c>
       <c r="I41">
-        <v>3065446681730.708</v>
+        <v>511907882162.8501</v>
       </c>
       <c r="J41">
-        <v>2430899218612.4521</v>
+        <v>405942950555.14008</v>
       </c>
       <c r="K41">
-        <v>247180551443.41281</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B42">
-        <v>28.001000000000001</v>
-      </c>
-      <c r="C42">
-        <v>10</v>
-      </c>
-      <c r="D42">
-        <v>37.975999999999999</v>
-      </c>
-      <c r="E42">
-        <v>9919.3920495248731</v>
-      </c>
-      <c r="F42">
-        <v>123054.2299165951</v>
-      </c>
-      <c r="G42">
-        <v>123054.2299165951</v>
-      </c>
-      <c r="H42">
-        <v>2948819312643.0649</v>
-      </c>
-      <c r="I42">
-        <v>2948819312643.0649</v>
-      </c>
-      <c r="J42">
-        <v>2338413714925.9512</v>
-      </c>
-      <c r="K42">
-        <v>237704098958.18051</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B43">
-        <v>28.001000000000001</v>
-      </c>
-      <c r="C43">
-        <v>10</v>
-      </c>
-      <c r="D43">
-        <v>37.975999999999999</v>
-      </c>
-      <c r="E43">
-        <v>9919.3920495248731</v>
-      </c>
-      <c r="F43">
-        <v>123054.2299165951</v>
-      </c>
-      <c r="G43">
-        <v>123054.2299165951</v>
-      </c>
-      <c r="H43">
-        <v>2948819312643.0649</v>
-      </c>
-      <c r="I43">
-        <v>2948819312643.0649</v>
-      </c>
-      <c r="J43">
-        <v>2338413714925.9512</v>
-      </c>
-      <c r="K43">
-        <v>237704098958.18051</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B44">
-        <v>28.001999999999999</v>
-      </c>
-      <c r="C44">
-        <v>10</v>
-      </c>
-      <c r="D44">
-        <v>36.456000000000003</v>
-      </c>
-      <c r="E44">
-        <v>9523.8185311774014</v>
-      </c>
-      <c r="F44">
-        <v>118182.8952025789</v>
-      </c>
-      <c r="G44">
-        <v>118182.8952025789</v>
-      </c>
-      <c r="H44">
-        <v>2832084716093.4321</v>
-      </c>
-      <c r="I44">
-        <v>2832084716093.4321</v>
-      </c>
-      <c r="J44">
-        <v>2245843179862.0918</v>
-      </c>
-      <c r="K44">
-        <v>228224743138.6868</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B45">
-        <v>41</v>
-      </c>
-      <c r="C45">
-        <v>9.9260000000000002</v>
-      </c>
-      <c r="D45">
-        <v>36.456000000000003</v>
-      </c>
-      <c r="E45">
-        <v>9453.0844057189461</v>
-      </c>
-      <c r="F45">
-        <v>115569.1673620746</v>
-      </c>
-      <c r="G45">
-        <v>115569.1673620746</v>
-      </c>
-      <c r="H45">
-        <v>2769450452002.7461</v>
-      </c>
-      <c r="I45">
-        <v>2769450452002.7461</v>
-      </c>
-      <c r="J45">
-        <v>2196174208438.178</v>
-      </c>
-      <c r="K45">
-        <v>226529700592.35431</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B46">
-        <v>41.000999999999998</v>
-      </c>
-      <c r="C46">
-        <v>9.9260000000000002</v>
-      </c>
-      <c r="D46">
-        <v>35.118000000000002</v>
-      </c>
-      <c r="E46">
-        <v>9107.3714150505875</v>
-      </c>
-      <c r="F46">
-        <v>111372.6561740015</v>
-      </c>
-      <c r="G46">
-        <v>111372.6561740015</v>
-      </c>
-      <c r="H46">
-        <v>2668887039875.4248</v>
-      </c>
-      <c r="I46">
-        <v>2668887039875.4248</v>
-      </c>
-      <c r="J46">
-        <v>2116427422621.2119</v>
-      </c>
-      <c r="K46">
-        <v>218245181285.65991</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B47">
-        <v>41.000999999999998</v>
-      </c>
-      <c r="C47">
-        <v>9.9260000000000002</v>
-      </c>
-      <c r="D47">
-        <v>35.118000000000002</v>
-      </c>
-      <c r="E47">
-        <v>9107.3714150505875</v>
-      </c>
-      <c r="F47">
-        <v>111372.6561740015</v>
-      </c>
-      <c r="G47">
-        <v>111372.6561740015</v>
-      </c>
-      <c r="H47">
-        <v>2668887039875.4248</v>
-      </c>
-      <c r="I47">
-        <v>2668887039875.4248</v>
-      </c>
-      <c r="J47">
-        <v>2116427422621.2119</v>
-      </c>
-      <c r="K47">
-        <v>218245181285.65991</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B48">
-        <v>41.002000000000002</v>
-      </c>
-      <c r="C48">
-        <v>9.9260000000000002</v>
-      </c>
-      <c r="D48">
-        <v>33.779000000000003</v>
-      </c>
-      <c r="E48">
-        <v>8761.3060592618385</v>
-      </c>
-      <c r="F48">
-        <v>107169.58508948211</v>
-      </c>
-      <c r="G48">
-        <v>107169.58508948211</v>
-      </c>
-      <c r="H48">
-        <v>2568166429175.2251</v>
-      </c>
-      <c r="I48">
-        <v>2568166429175.2251</v>
-      </c>
-      <c r="J48">
-        <v>2036555978335.9529</v>
-      </c>
-      <c r="K48">
-        <v>209952218050.84689</v>
-      </c>
-    </row>
-    <row r="49" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B49">
-        <v>54</v>
-      </c>
-      <c r="C49">
-        <v>9.4429999999999996</v>
-      </c>
-      <c r="D49">
-        <v>33.779000000000003</v>
-      </c>
-      <c r="E49">
-        <v>8333.5243885306409</v>
-      </c>
-      <c r="F49">
-        <v>92225.636090311411</v>
-      </c>
-      <c r="G49">
-        <v>92225.636090311411</v>
-      </c>
-      <c r="H49">
-        <v>2210055981076.2378</v>
-      </c>
-      <c r="I49">
-        <v>2210055981076.2378</v>
-      </c>
-      <c r="J49">
-        <v>1752574392993.457</v>
-      </c>
-      <c r="K49">
-        <v>199701039744.32401</v>
-      </c>
-    </row>
-    <row r="50" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B50">
-        <v>54.000999999999998</v>
-      </c>
-      <c r="C50">
-        <v>9.4429999999999996</v>
-      </c>
-      <c r="D50">
-        <v>32.985999999999997</v>
-      </c>
-      <c r="E50">
-        <v>8138.5713878846082</v>
-      </c>
-      <c r="F50">
-        <v>90083.25410621558</v>
-      </c>
-      <c r="G50">
-        <v>90083.25410621558</v>
-      </c>
-      <c r="H50">
-        <v>2158716848938.7871</v>
-      </c>
-      <c r="I50">
-        <v>2158716848938.7871</v>
-      </c>
-      <c r="J50">
-        <v>1711862461208.458</v>
-      </c>
-      <c r="K50">
-        <v>195029268820.62329</v>
-      </c>
-    </row>
-    <row r="51" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B51">
-        <v>54.000999999999998</v>
-      </c>
-      <c r="C51">
-        <v>9.4429999999999996</v>
-      </c>
-      <c r="D51">
-        <v>32.985999999999997</v>
-      </c>
-      <c r="E51">
-        <v>8138.5713878846082</v>
-      </c>
-      <c r="F51">
-        <v>90083.25410621558</v>
-      </c>
-      <c r="G51">
-        <v>90083.25410621558</v>
-      </c>
-      <c r="H51">
-        <v>2158716848938.7871</v>
-      </c>
-      <c r="I51">
-        <v>2158716848938.7871</v>
-      </c>
-      <c r="J51">
-        <v>1711862461208.458</v>
-      </c>
-      <c r="K51">
-        <v>195029268820.62329</v>
-      </c>
-    </row>
-    <row r="52" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B52">
-        <v>54.002000000000002</v>
-      </c>
-      <c r="C52">
-        <v>9.4429999999999996</v>
-      </c>
-      <c r="D52">
-        <v>32.192</v>
-      </c>
-      <c r="E52">
-        <v>7943.339505959193</v>
-      </c>
-      <c r="F52">
-        <v>87937.081105321893</v>
-      </c>
-      <c r="G52">
-        <v>87937.081105321893</v>
-      </c>
-      <c r="H52">
-        <v>2107286870484.5891</v>
-      </c>
-      <c r="I52">
-        <v>2107286870484.5891</v>
-      </c>
-      <c r="J52">
-        <v>1671078488294.2791</v>
-      </c>
-      <c r="K52">
-        <v>190350814904.366</v>
-      </c>
-    </row>
-    <row r="53" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B53">
-        <v>67</v>
-      </c>
-      <c r="C53">
-        <v>8.8330000000000002</v>
-      </c>
-      <c r="D53">
-        <v>32.192</v>
-      </c>
-      <c r="E53">
-        <v>7428.4594766741811</v>
-      </c>
-      <c r="F53">
-        <v>71921.655457150788</v>
-      </c>
-      <c r="G53">
-        <v>71921.655457150788</v>
-      </c>
-      <c r="H53">
-        <v>1723500010954.967</v>
-      </c>
-      <c r="I53">
-        <v>1723500010954.967</v>
-      </c>
-      <c r="J53">
-        <v>1366735508687.2891</v>
-      </c>
-      <c r="K53">
-        <v>178012448518.43231</v>
-      </c>
-    </row>
-    <row r="54" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B54">
-        <v>67.001000000000005</v>
-      </c>
-      <c r="C54">
-        <v>8.8330000000000002</v>
-      </c>
-      <c r="D54">
-        <v>31.45</v>
-      </c>
-      <c r="E54">
-        <v>7257.8512541112013</v>
-      </c>
-      <c r="F54">
-        <v>70281.648937049016</v>
-      </c>
-      <c r="G54">
-        <v>70281.648937049016</v>
-      </c>
-      <c r="H54">
-        <v>1684199591110.688</v>
-      </c>
-      <c r="I54">
-        <v>1684199591110.688</v>
-      </c>
-      <c r="J54">
-        <v>1335570275750.7759</v>
-      </c>
-      <c r="K54">
-        <v>173924065519.0798</v>
-      </c>
-    </row>
-    <row r="55" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B55">
-        <v>67.001000000000005</v>
-      </c>
-      <c r="C55">
-        <v>8.8330000000000002</v>
-      </c>
-      <c r="D55">
-        <v>31.45</v>
-      </c>
-      <c r="E55">
-        <v>7257.8512541112013</v>
-      </c>
-      <c r="F55">
-        <v>70281.648937049016</v>
-      </c>
-      <c r="G55">
-        <v>70281.648937049016</v>
-      </c>
-      <c r="H55">
-        <v>1684199591110.688</v>
-      </c>
-      <c r="I55">
-        <v>1684199591110.688</v>
-      </c>
-      <c r="J55">
-        <v>1335570275750.7759</v>
-      </c>
-      <c r="K55">
-        <v>173924065519.0798</v>
-      </c>
-    </row>
-    <row r="56" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B56">
-        <v>67.001999999999995</v>
-      </c>
-      <c r="C56">
-        <v>8.8330000000000002</v>
-      </c>
-      <c r="D56">
-        <v>30.707999999999998</v>
-      </c>
-      <c r="E56">
-        <v>7087.214160266677</v>
-      </c>
-      <c r="F56">
-        <v>68640.809682709922</v>
-      </c>
-      <c r="G56">
-        <v>68640.809682709922</v>
-      </c>
-      <c r="H56">
-        <v>1644879215976.7529</v>
-      </c>
-      <c r="I56">
-        <v>1644879215976.7529</v>
-      </c>
-      <c r="J56">
-        <v>1304389218269.5649</v>
-      </c>
-      <c r="K56">
-        <v>169834990660.59619</v>
-      </c>
-    </row>
-    <row r="57" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B57">
-        <v>80</v>
-      </c>
-      <c r="C57">
-        <v>8.1509999999999998</v>
-      </c>
-      <c r="D57">
-        <v>30.707999999999998</v>
-      </c>
-      <c r="E57">
-        <v>6538.0980826244668</v>
-      </c>
-      <c r="F57">
-        <v>53890.34303307574</v>
-      </c>
-      <c r="G57">
-        <v>53890.34303307574</v>
-      </c>
-      <c r="H57">
-        <v>1291405296742.769</v>
-      </c>
-      <c r="I57">
-        <v>1291405296742.769</v>
-      </c>
-      <c r="J57">
-        <v>1024084400317.016</v>
-      </c>
-      <c r="K57">
-        <v>156676206149.63971</v>
-      </c>
-    </row>
-    <row r="58" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B58">
-        <v>80.001000000000005</v>
-      </c>
-      <c r="C58">
-        <v>8.1509999999999998</v>
-      </c>
-      <c r="D58">
-        <v>29.904</v>
-      </c>
-      <c r="E58">
-        <v>6367.5473254292383</v>
-      </c>
-      <c r="F58">
-        <v>52494.931303291327</v>
-      </c>
-      <c r="G58">
-        <v>52494.931303291327</v>
-      </c>
-      <c r="H58">
-        <v>1257966242590.2549</v>
-      </c>
-      <c r="I58">
-        <v>1257966242590.2549</v>
-      </c>
-      <c r="J58">
-        <v>997567230374.0719</v>
-      </c>
-      <c r="K58">
-        <v>152589200225.95831</v>
-      </c>
-    </row>
-    <row r="59" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B59">
-        <v>80.001000000000005</v>
-      </c>
-      <c r="C59">
-        <v>8.1509999999999998</v>
-      </c>
-      <c r="D59">
-        <v>29.904</v>
-      </c>
-      <c r="E59">
-        <v>6367.5473254292383</v>
-      </c>
-      <c r="F59">
-        <v>52494.931303291327</v>
-      </c>
-      <c r="G59">
-        <v>52494.931303291327</v>
-      </c>
-      <c r="H59">
-        <v>1257966242590.2549</v>
-      </c>
-      <c r="I59">
-        <v>1257966242590.2549</v>
-      </c>
-      <c r="J59">
-        <v>997567230374.0719</v>
-      </c>
-      <c r="K59">
-        <v>152589200225.95831</v>
-      </c>
-    </row>
-    <row r="60" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B60">
-        <v>80.001999999999995</v>
-      </c>
-      <c r="C60">
-        <v>8.1509999999999998</v>
-      </c>
-      <c r="D60">
-        <v>29.100999999999999</v>
-      </c>
-      <c r="E60">
-        <v>6197.1748615481274</v>
-      </c>
-      <c r="F60">
-        <v>51100.424514406717</v>
-      </c>
-      <c r="G60">
-        <v>51100.424514406717</v>
-      </c>
-      <c r="H60">
-        <v>1224548874057.1941</v>
-      </c>
-      <c r="I60">
-        <v>1224548874057.1941</v>
-      </c>
-      <c r="J60">
-        <v>971067257127.3551</v>
-      </c>
-      <c r="K60">
-        <v>148506466847.54681</v>
-      </c>
-    </row>
-    <row r="61" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B61">
-        <v>93</v>
-      </c>
-      <c r="C61">
-        <v>7.39</v>
-      </c>
-      <c r="D61">
-        <v>29.100999999999999</v>
-      </c>
-      <c r="E61">
-        <v>5616.5163148661431</v>
-      </c>
-      <c r="F61">
-        <v>38040.441011391602</v>
-      </c>
-      <c r="G61">
-        <v>38040.441011391602</v>
-      </c>
-      <c r="H61">
-        <v>911584975111.22949</v>
-      </c>
-      <c r="I61">
-        <v>911584975111.22949</v>
-      </c>
-      <c r="J61">
-        <v>722886885263.20496</v>
-      </c>
-      <c r="K61">
-        <v>134591812002.54359</v>
-      </c>
-    </row>
-    <row r="62" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B62">
-        <v>93.001000000000005</v>
-      </c>
-      <c r="C62">
-        <v>7.39</v>
-      </c>
-      <c r="D62">
-        <v>28.157</v>
-      </c>
-      <c r="E62">
-        <v>5435.0204844990558</v>
-      </c>
-      <c r="F62">
-        <v>36820.582440753249</v>
-      </c>
-      <c r="G62">
-        <v>36820.582440753249</v>
-      </c>
-      <c r="H62">
-        <v>882352802318.55383</v>
-      </c>
-      <c r="I62">
-        <v>882352802318.55383</v>
-      </c>
-      <c r="J62">
-        <v>699705772238.61316</v>
-      </c>
-      <c r="K62">
-        <v>130242522993.02789</v>
-      </c>
-    </row>
-    <row r="63" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B63">
-        <v>93.001000000000005</v>
-      </c>
-      <c r="C63">
-        <v>7.39</v>
-      </c>
-      <c r="D63">
-        <v>28.157</v>
-      </c>
-      <c r="E63">
-        <v>5435.0204844990558</v>
-      </c>
-      <c r="F63">
-        <v>36820.582440753249</v>
-      </c>
-      <c r="G63">
-        <v>36820.582440753249</v>
-      </c>
-      <c r="H63">
-        <v>882352802318.55383</v>
-      </c>
-      <c r="I63">
-        <v>882352802318.55383</v>
-      </c>
-      <c r="J63">
-        <v>699705772238.61316</v>
-      </c>
-      <c r="K63">
-        <v>130242522993.02789</v>
-      </c>
-    </row>
-    <row r="64" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B64">
-        <v>93.001999999999995</v>
-      </c>
-      <c r="C64">
-        <v>7.39</v>
-      </c>
-      <c r="D64">
-        <v>27.213000000000001</v>
-      </c>
-      <c r="E64">
-        <v>5253.4779234371445</v>
-      </c>
-      <c r="F64">
-        <v>35599.7813771168</v>
-      </c>
-      <c r="G64">
-        <v>35599.7813771168</v>
-      </c>
-      <c r="H64">
-        <v>853098044023.88684</v>
-      </c>
-      <c r="I64">
-        <v>853098044023.88684</v>
-      </c>
-      <c r="J64">
-        <v>676506748910.94226</v>
-      </c>
-      <c r="K64">
-        <v>125892114148.985</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B65">
-        <v>106</v>
-      </c>
-      <c r="C65">
-        <v>6.9089999999999998</v>
-      </c>
-      <c r="D65">
-        <v>27.213000000000001</v>
-      </c>
-      <c r="E65">
-        <v>4910.275969995676</v>
-      </c>
-      <c r="F65">
-        <v>29068.669776437349</v>
-      </c>
-      <c r="G65">
-        <v>29068.669776437349</v>
-      </c>
-      <c r="H65">
-        <v>696589258960.87573</v>
-      </c>
-      <c r="I65">
-        <v>696589258960.87573</v>
-      </c>
-      <c r="J65">
-        <v>552395282355.97449</v>
-      </c>
-      <c r="K65">
-        <v>117667768272.1226</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B66">
-        <v>106.001</v>
-      </c>
-      <c r="C66">
-        <v>6.9089999999999998</v>
-      </c>
-      <c r="D66">
-        <v>25.611000000000001</v>
-      </c>
-      <c r="E66">
-        <v>4622.2890770266577</v>
-      </c>
-      <c r="F66">
-        <v>27376.48932322409</v>
-      </c>
-      <c r="G66">
-        <v>27376.48932322409</v>
-      </c>
-      <c r="H66">
-        <v>656038565138.36768</v>
-      </c>
-      <c r="I66">
-        <v>656038565138.36768</v>
-      </c>
-      <c r="J66">
-        <v>520238582154.72559</v>
-      </c>
-      <c r="K66">
-        <v>110766572658.1993</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B67">
-        <v>106.001</v>
-      </c>
-      <c r="C67">
-        <v>6.9089999999999998</v>
-      </c>
-      <c r="D67">
-        <v>25.611000000000001</v>
-      </c>
-      <c r="E67">
-        <v>4622.2890770266577</v>
-      </c>
-      <c r="F67">
-        <v>27376.48932322409</v>
-      </c>
-      <c r="G67">
-        <v>27376.48932322409</v>
-      </c>
-      <c r="H67">
-        <v>656038565138.36768</v>
-      </c>
-      <c r="I67">
-        <v>656038565138.36768</v>
-      </c>
-      <c r="J67">
-        <v>520238582154.72559</v>
-      </c>
-      <c r="K67">
-        <v>110766572658.1993</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B68">
-        <v>106.002</v>
-      </c>
-      <c r="C68">
-        <v>6.9089999999999998</v>
-      </c>
-      <c r="D68">
-        <v>24.009</v>
-      </c>
-      <c r="E68">
-        <v>4334.1676032059768</v>
-      </c>
-      <c r="F68">
-        <v>25681.93541283693</v>
-      </c>
-      <c r="G68">
-        <v>25681.93541283693</v>
-      </c>
-      <c r="H68">
-        <v>615430994795.99658</v>
-      </c>
-      <c r="I68">
-        <v>615430994795.99658</v>
-      </c>
-      <c r="J68">
-        <v>488036778873.22522</v>
-      </c>
-      <c r="K68">
-        <v>103862152005.8945</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B69">
-        <v>119</v>
-      </c>
-      <c r="C69">
-        <v>6.7480000000000002</v>
-      </c>
-      <c r="D69">
-        <v>24.009</v>
-      </c>
-      <c r="E69">
-        <v>4232.8165652574853</v>
-      </c>
-      <c r="F69">
-        <v>23922.096893685812</v>
-      </c>
-      <c r="G69">
-        <v>23922.096893685812</v>
-      </c>
-      <c r="H69">
-        <v>573258971811.30627</v>
-      </c>
-      <c r="I69">
-        <v>573258971811.30627</v>
-      </c>
-      <c r="J69">
-        <v>454594364646.36578</v>
-      </c>
-      <c r="K69">
-        <v>101433418769.6498</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B70">
-        <v>119.001</v>
-      </c>
-      <c r="C70">
-        <v>6.7480000000000002</v>
-      </c>
-      <c r="D70">
-        <v>22.417999999999999</v>
-      </c>
-      <c r="E70">
-        <v>3953.2564663697899</v>
-      </c>
-      <c r="F70">
-        <v>22352.678535921561</v>
-      </c>
-      <c r="G70">
-        <v>22352.678535921561</v>
-      </c>
-      <c r="H70">
-        <v>535650096715.11072</v>
-      </c>
-      <c r="I70">
-        <v>535650096715.11072</v>
-      </c>
-      <c r="J70">
-        <v>424770526695.08282</v>
-      </c>
-      <c r="K70">
-        <v>94734159270.783371</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B71">
-        <v>119.001</v>
-      </c>
-      <c r="C71">
-        <v>6.7480000000000002</v>
-      </c>
-      <c r="D71">
-        <v>22.417999999999999</v>
-      </c>
-      <c r="E71">
-        <v>3953.2564663697899</v>
-      </c>
-      <c r="F71">
-        <v>22352.678535921561</v>
-      </c>
-      <c r="G71">
-        <v>22352.678535921561</v>
-      </c>
-      <c r="H71">
-        <v>535650096715.11072</v>
-      </c>
-      <c r="I71">
-        <v>535650096715.11072</v>
-      </c>
-      <c r="J71">
-        <v>424770526695.08282</v>
-      </c>
-      <c r="K71">
-        <v>94734159270.783371</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B72">
-        <v>119.002</v>
-      </c>
-      <c r="C72">
-        <v>6.7480000000000002</v>
-      </c>
-      <c r="D72">
-        <v>20.826000000000001</v>
-      </c>
-      <c r="E72">
-        <v>3673.3877898387768</v>
-      </c>
-      <c r="F72">
-        <v>20780.03502692196</v>
-      </c>
-      <c r="G72">
-        <v>20780.03502692196</v>
-      </c>
-      <c r="H72">
-        <v>497963935464.22137</v>
-      </c>
-      <c r="I72">
-        <v>497963935464.22137</v>
-      </c>
-      <c r="J72">
-        <v>394885400823.12762</v>
-      </c>
-      <c r="K72">
-        <v>88027505148.305237</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B73">
-        <v>132</v>
-      </c>
-      <c r="C73">
-        <v>6.5720000000000001</v>
-      </c>
-      <c r="D73">
-        <v>20.826000000000001</v>
-      </c>
-      <c r="E73">
-        <v>3577.282612388075</v>
-      </c>
-      <c r="F73">
-        <v>19191.367526978469</v>
-      </c>
-      <c r="G73">
-        <v>19191.367526978469</v>
-      </c>
-      <c r="H73">
-        <v>459893782098.69342</v>
-      </c>
-      <c r="I73">
-        <v>459893782098.69342</v>
-      </c>
-      <c r="J73">
-        <v>364695769204.26392</v>
-      </c>
-      <c r="K73">
-        <v>85724481485.455917</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B74">
-        <v>132.001</v>
-      </c>
-      <c r="C74">
-        <v>6.5720000000000001</v>
-      </c>
-      <c r="D74">
-        <v>22.411999999999999</v>
-      </c>
-      <c r="E74">
-        <v>3848.7778857902158</v>
-      </c>
-      <c r="F74">
-        <v>20637.919313358329</v>
-      </c>
-      <c r="G74">
-        <v>20637.919313358329</v>
-      </c>
-      <c r="H74">
-        <v>494558334851.62543</v>
-      </c>
-      <c r="I74">
-        <v>494558334851.62543</v>
-      </c>
-      <c r="J74">
-        <v>392184759537.33893</v>
-      </c>
-      <c r="K74">
-        <v>92230478930.990097</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B75">
-        <v>132.001</v>
-      </c>
-      <c r="C75">
-        <v>6.5720000000000001</v>
-      </c>
-      <c r="D75">
-        <v>22.411999999999999</v>
-      </c>
-      <c r="E75">
-        <v>3848.7778857902158</v>
-      </c>
-      <c r="F75">
-        <v>20637.919313358329</v>
-      </c>
-      <c r="G75">
-        <v>20637.919313358329</v>
-      </c>
-      <c r="H75">
-        <v>494558334851.62543</v>
-      </c>
-      <c r="I75">
-        <v>494558334851.62543</v>
-      </c>
-      <c r="J75">
-        <v>392184759537.33893</v>
-      </c>
-      <c r="K75">
-        <v>92230478930.990097</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B76">
-        <v>132.00200000000001</v>
-      </c>
-      <c r="C76">
-        <v>6.5720000000000001</v>
-      </c>
-      <c r="D76">
-        <v>23.998000000000001</v>
-      </c>
-      <c r="E76">
-        <v>4120.1412531729766</v>
-      </c>
-      <c r="F76">
-        <v>22082.363701823171</v>
-      </c>
-      <c r="G76">
-        <v>22082.363701823171</v>
-      </c>
-      <c r="H76">
-        <v>529172386815.79602</v>
-      </c>
-      <c r="I76">
-        <v>529172386815.79602</v>
-      </c>
-      <c r="J76">
-        <v>419633702744.92621</v>
-      </c>
-      <c r="K76">
-        <v>98733315436.687683</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A77" t="s">
-        <v>195</v>
-      </c>
-      <c r="B77">
-        <v>144.386</v>
-      </c>
-      <c r="C77">
-        <v>6.5</v>
-      </c>
-      <c r="D77">
-        <v>23.998000000000001</v>
-      </c>
-      <c r="E77">
-        <v>4074.8373314227201</v>
-      </c>
-      <c r="F77">
-        <v>21361.915922655739</v>
-      </c>
-      <c r="G77">
-        <v>21361.915922655739</v>
-      </c>
-      <c r="H77">
-        <v>511907882162.8501</v>
-      </c>
-      <c r="I77">
-        <v>511907882162.8501</v>
-      </c>
-      <c r="J77">
-        <v>405942950555.14008</v>
-      </c>
-      <c r="K77">
         <v>97647671493.475189</v>
       </c>
     </row>
@@ -19293,16 +18155,17 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="15" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="13" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="17" x14ac:dyDescent="0.2">
@@ -19365,52 +18228,52 @@
       <c r="A3" t="s">
         <v>264</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="6">
         <v>48092.001786537301</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="5">
         <v>-7.0885261800196808</v>
       </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
+      <c r="D3" s="5">
+        <v>0</v>
+      </c>
+      <c r="E3" s="5">
         <v>5.094493537559762</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="6">
         <v>59002.874691857964</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="6">
         <v>29771.954855978249</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="6">
         <v>29771.954855978249</v>
       </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
-      <c r="J3">
-        <v>0</v>
-      </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
-      <c r="L3">
+      <c r="I3" s="6">
+        <v>0</v>
+      </c>
+      <c r="J3" s="6">
+        <v>0</v>
+      </c>
+      <c r="K3" s="6">
+        <v>0</v>
+      </c>
+      <c r="L3" s="6">
         <v>1306856.7851224421</v>
       </c>
-      <c r="M3">
+      <c r="M3" s="6">
         <v>3694433.844065466</v>
       </c>
-      <c r="N3">
+      <c r="N3" s="6">
         <v>2446579.9336348828</v>
       </c>
-      <c r="O3">
-        <v>0</v>
-      </c>
-      <c r="P3">
+      <c r="O3" s="6">
+        <v>0</v>
+      </c>
+      <c r="P3" s="6">
         <v>1733681.3241244019</v>
       </c>
-      <c r="Q3">
+      <c r="Q3" s="6">
         <v>0</v>
       </c>
     </row>
@@ -19418,52 +18281,52 @@
       <c r="A4" t="s">
         <v>265</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="6">
         <v>13479.28387693245</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="5">
         <v>-5.8950999055777533</v>
       </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
+      <c r="D4" s="5">
+        <v>0</v>
+      </c>
+      <c r="E4" s="5">
         <v>4.9690593816385773</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="6">
         <v>16537.3964065115</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="6">
         <v>8344.5191750634949</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="6">
         <v>8344.5191750634949</v>
       </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
-      <c r="L4">
+      <c r="I4" s="6">
+        <v>0</v>
+      </c>
+      <c r="J4" s="6">
+        <v>0</v>
+      </c>
+      <c r="K4" s="6">
+        <v>0</v>
+      </c>
+      <c r="L4" s="6">
         <v>349272.30654858239</v>
       </c>
-      <c r="M4">
+      <c r="M4" s="6">
         <v>809603.75452328555</v>
       </c>
-      <c r="N4">
+      <c r="N4" s="6">
         <v>476868.84438121459</v>
       </c>
-      <c r="O4">
-        <v>0</v>
-      </c>
-      <c r="P4">
+      <c r="O4" s="6">
+        <v>0</v>
+      </c>
+      <c r="P4" s="6">
         <v>393998.33316090098</v>
       </c>
-      <c r="Q4">
+      <c r="Q4" s="6">
         <v>0</v>
       </c>
     </row>
@@ -19471,52 +18334,52 @@
       <c r="A5" t="s">
         <v>266</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="6">
         <v>15734.038486973781</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="5">
         <v>-6.9890739904828534</v>
       </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
+      <c r="D5" s="5">
+        <v>0</v>
+      </c>
+      <c r="E5" s="5">
         <v>5.0840406912329961</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="6">
         <v>33120.151015079799</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="6">
         <v>22906.137697285991</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="6">
         <v>22906.137697285991</v>
       </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-      <c r="J5">
-        <v>0</v>
-      </c>
-      <c r="K5">
-        <v>0</v>
-      </c>
-      <c r="L5">
+      <c r="I5" s="6">
+        <v>0</v>
+      </c>
+      <c r="J5" s="6">
+        <v>0</v>
+      </c>
+      <c r="K5" s="6">
+        <v>0</v>
+      </c>
+      <c r="L5" s="6">
         <v>439693.63450568088</v>
       </c>
-      <c r="M5">
+      <c r="M5" s="6">
         <v>1198154.2421317161</v>
       </c>
-      <c r="N5">
+      <c r="N5" s="6">
         <v>791580.75864111481</v>
       </c>
-      <c r="O5">
-        <v>0</v>
-      </c>
-      <c r="P5">
+      <c r="O5" s="6">
+        <v>0</v>
+      </c>
+      <c r="P5" s="6">
         <v>558011.63821907982</v>
       </c>
-      <c r="Q5">
+      <c r="Q5" s="6">
         <v>0</v>
       </c>
     </row>
@@ -19524,52 +18387,52 @@
       <c r="A6" t="s">
         <v>267</v>
       </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-      <c r="C6">
+      <c r="B6" s="6">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5">
         <v>-5.0000301997463072</v>
       </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
-      <c r="E6">
+      <c r="D6" s="5">
+        <v>0</v>
+      </c>
+      <c r="E6" s="5">
         <v>4.8749837646976886</v>
       </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-      <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6">
-        <v>0</v>
-      </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-      <c r="J6">
-        <v>0</v>
-      </c>
-      <c r="K6">
-        <v>0</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6">
-        <v>0</v>
-      </c>
-      <c r="N6">
-        <v>0</v>
-      </c>
-      <c r="O6">
-        <v>0</v>
-      </c>
-      <c r="P6">
-        <v>0</v>
-      </c>
-      <c r="Q6">
+      <c r="F6" s="6">
+        <v>0</v>
+      </c>
+      <c r="G6" s="6">
+        <v>0</v>
+      </c>
+      <c r="H6" s="6">
+        <v>0</v>
+      </c>
+      <c r="I6" s="6">
+        <v>0</v>
+      </c>
+      <c r="J6" s="6">
+        <v>0</v>
+      </c>
+      <c r="K6" s="6">
+        <v>0</v>
+      </c>
+      <c r="L6" s="6">
+        <v>0</v>
+      </c>
+      <c r="M6" s="6">
+        <v>0</v>
+      </c>
+      <c r="N6" s="6">
+        <v>0</v>
+      </c>
+      <c r="O6" s="6">
+        <v>0</v>
+      </c>
+      <c r="P6" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="6">
         <v>0</v>
       </c>
     </row>
@@ -19577,52 +18440,52 @@
       <c r="A7" t="s">
         <v>268</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="6">
         <v>24290.364248076799</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="5">
         <v>-7.585787127703818</v>
       </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-      <c r="E7">
+      <c r="D7" s="5">
+        <v>0</v>
+      </c>
+      <c r="E7" s="5">
         <v>5.1467577691935888</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="6">
         <v>17686.462299954401</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="6">
         <v>8843.2311499772022</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="6">
         <v>8843.2311499772022</v>
       </c>
-      <c r="I7">
-        <v>0</v>
-      </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
-      <c r="K7">
-        <v>0</v>
-      </c>
-      <c r="L7">
+      <c r="I7" s="6">
+        <v>0</v>
+      </c>
+      <c r="J7" s="6">
+        <v>0</v>
+      </c>
+      <c r="K7" s="6">
+        <v>0</v>
+      </c>
+      <c r="L7" s="6">
         <v>661020.10433958611</v>
       </c>
-      <c r="M7">
+      <c r="M7" s="6">
         <v>2050042.257015147</v>
       </c>
-      <c r="N7">
+      <c r="N7" s="6">
         <v>1406708.6149755151</v>
       </c>
-      <c r="O7">
-        <v>0</v>
-      </c>
-      <c r="P7">
+      <c r="O7" s="6">
+        <v>0</v>
+      </c>
+      <c r="P7" s="6">
         <v>947430.16808027821</v>
       </c>
-      <c r="Q7">
+      <c r="Q7" s="6">
         <v>0</v>
       </c>
     </row>
@@ -19630,52 +18493,52 @@
       <c r="A8" t="s">
         <v>269</v>
       </c>
-      <c r="B8">
-        <v>0</v>
-      </c>
-      <c r="C8">
+      <c r="B8" s="6">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5">
         <v>-5.0000301997463072</v>
       </c>
-      <c r="D8">
-        <v>0</v>
-      </c>
-      <c r="E8">
+      <c r="D8" s="5">
+        <v>0</v>
+      </c>
+      <c r="E8" s="5">
         <v>4.8749837646976886</v>
       </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8">
-        <v>0</v>
-      </c>
-      <c r="I8">
-        <v>0</v>
-      </c>
-      <c r="J8">
-        <v>0</v>
-      </c>
-      <c r="K8">
-        <v>0</v>
-      </c>
-      <c r="L8">
-        <v>0</v>
-      </c>
-      <c r="M8">
-        <v>0</v>
-      </c>
-      <c r="N8">
-        <v>0</v>
-      </c>
-      <c r="O8">
-        <v>0</v>
-      </c>
-      <c r="P8">
-        <v>0</v>
-      </c>
-      <c r="Q8">
+      <c r="F8" s="6">
+        <v>0</v>
+      </c>
+      <c r="G8" s="6">
+        <v>0</v>
+      </c>
+      <c r="H8" s="6">
+        <v>0</v>
+      </c>
+      <c r="I8" s="6">
+        <v>0</v>
+      </c>
+      <c r="J8" s="6">
+        <v>0</v>
+      </c>
+      <c r="K8" s="6">
+        <v>0</v>
+      </c>
+      <c r="L8" s="6">
+        <v>0</v>
+      </c>
+      <c r="M8" s="6">
+        <v>0</v>
+      </c>
+      <c r="N8" s="6">
+        <v>0</v>
+      </c>
+      <c r="O8" s="6">
+        <v>0</v>
+      </c>
+      <c r="P8" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="6">
         <v>0</v>
       </c>
     </row>
@@ -19683,52 +18546,52 @@
       <c r="A9" t="s">
         <v>270</v>
       </c>
-      <c r="B9">
-        <v>184419.5</v>
-      </c>
-      <c r="C9">
-        <v>-6.5166760901829237</v>
-      </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-      <c r="E9">
-        <v>5.0343896711808611</v>
-      </c>
-      <c r="F9">
-        <v>2598976.1566397501</v>
-      </c>
-      <c r="G9">
-        <v>1370528.006549042</v>
-      </c>
-      <c r="H9">
-        <v>1370528.006549042</v>
-      </c>
-      <c r="I9">
-        <v>0</v>
-      </c>
-      <c r="J9">
-        <v>0</v>
-      </c>
-      <c r="K9">
-        <v>0</v>
-      </c>
-      <c r="L9">
-        <v>7259680.7501828391</v>
-      </c>
-      <c r="M9">
-        <v>13876410.181178899</v>
-      </c>
-      <c r="N9">
-        <v>9215705.5876358133</v>
-      </c>
-      <c r="O9">
-        <v>0</v>
-      </c>
-      <c r="P9">
-        <v>5922635.9457165301</v>
-      </c>
-      <c r="Q9">
+      <c r="B9" s="6">
+        <v>130349.249629283</v>
+      </c>
+      <c r="C9" s="5">
+        <v>-6.5166760901829202</v>
+      </c>
+      <c r="D9" s="5">
+        <v>0</v>
+      </c>
+      <c r="E9" s="5">
+        <v>5.0343896711808602</v>
+      </c>
+      <c r="F9" s="6">
+        <v>1836783.8456006399</v>
+      </c>
+      <c r="G9" s="6">
+        <v>972876.63394495798</v>
+      </c>
+      <c r="H9" s="6">
+        <v>972876.63394495798</v>
+      </c>
+      <c r="I9" s="6">
+        <v>0</v>
+      </c>
+      <c r="J9" s="6">
+        <v>0</v>
+      </c>
+      <c r="K9" s="6">
+        <v>0</v>
+      </c>
+      <c r="L9" s="7">
+        <v>5131056.6994807497</v>
+      </c>
+      <c r="M9" s="7">
+        <v>9812139.0623499602</v>
+      </c>
+      <c r="N9" s="7">
+        <v>6517866.20846985</v>
+      </c>
+      <c r="O9" s="6">
+        <v>0</v>
+      </c>
+      <c r="P9" s="7">
+        <v>4186623.0819099899</v>
+      </c>
+      <c r="Q9" s="6">
         <v>0</v>
       </c>
     </row>
@@ -19736,52 +18599,52 @@
       <c r="A10" t="s">
         <v>271</v>
       </c>
-      <c r="B10">
-        <v>184419.5</v>
-      </c>
-      <c r="C10">
-        <v>-6.5166760901829237</v>
-      </c>
-      <c r="D10">
-        <v>0</v>
-      </c>
-      <c r="E10">
-        <v>5.0343896711808611</v>
-      </c>
-      <c r="F10">
-        <v>2598976.1566397501</v>
-      </c>
-      <c r="G10">
-        <v>1370528.006549042</v>
-      </c>
-      <c r="H10">
-        <v>1370528.006549042</v>
-      </c>
-      <c r="I10">
-        <v>0</v>
-      </c>
-      <c r="J10">
-        <v>0</v>
-      </c>
-      <c r="K10">
-        <v>0</v>
-      </c>
-      <c r="L10">
-        <v>7259680.7501828391</v>
-      </c>
-      <c r="M10">
-        <v>13876410.181178899</v>
-      </c>
-      <c r="N10">
-        <v>9215705.5876358133</v>
-      </c>
-      <c r="O10">
-        <v>0</v>
-      </c>
-      <c r="P10">
-        <v>5922635.9457165301</v>
-      </c>
-      <c r="Q10">
+      <c r="B10" s="6">
+        <v>238490.15752252701</v>
+      </c>
+      <c r="C10" s="5">
+        <v>-6.5166760901829202</v>
+      </c>
+      <c r="D10" s="5">
+        <v>0</v>
+      </c>
+      <c r="E10" s="5">
+        <v>5.0343896711808602</v>
+      </c>
+      <c r="F10" s="6">
+        <v>3360624.39882062</v>
+      </c>
+      <c r="G10" s="6">
+        <v>1779998.7521170501</v>
+      </c>
+      <c r="H10" s="6">
+        <v>1779998.7521170501</v>
+      </c>
+      <c r="I10" s="6">
+        <v>0</v>
+      </c>
+      <c r="J10" s="6">
+        <v>0</v>
+      </c>
+      <c r="K10" s="6">
+        <v>0</v>
+      </c>
+      <c r="L10" s="6">
+        <v>9387906.1367551591</v>
+      </c>
+      <c r="M10" s="7">
+        <v>17952528.282809999</v>
+      </c>
+      <c r="N10" s="7">
+        <v>11925246.544875501</v>
+      </c>
+      <c r="O10" s="6">
+        <v>0</v>
+      </c>
+      <c r="P10" s="7">
+        <v>7659947.4191974998</v>
+      </c>
+      <c r="Q10" s="6">
         <v>0</v>
       </c>
     </row>
@@ -19789,52 +18652,52 @@
       <c r="A11" t="s">
         <v>272</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="6">
         <v>368839</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="5">
         <v>-6.5166760901829237</v>
       </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
-      <c r="E11">
+      <c r="D11" s="5">
+        <v>0</v>
+      </c>
+      <c r="E11" s="5">
         <v>5.0343896711808611</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="6">
         <v>5197952.3132795002</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="6">
         <v>2741056.013098083</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="6">
         <v>2741056.013098083</v>
       </c>
-      <c r="I11">
-        <v>0</v>
-      </c>
-      <c r="J11">
-        <v>0</v>
-      </c>
-      <c r="K11">
-        <v>0</v>
-      </c>
-      <c r="L11">
+      <c r="I11" s="6">
+        <v>0</v>
+      </c>
+      <c r="J11" s="6">
+        <v>0</v>
+      </c>
+      <c r="K11" s="6">
+        <v>0</v>
+      </c>
+      <c r="L11" s="6">
         <v>14519361.50036568</v>
       </c>
-      <c r="M11">
+      <c r="M11" s="6">
         <v>27752820.362357799</v>
       </c>
-      <c r="N11">
+      <c r="N11" s="6">
         <v>18431411.17527163</v>
       </c>
-      <c r="O11">
-        <v>0</v>
-      </c>
-      <c r="P11">
+      <c r="O11" s="6">
+        <v>0</v>
+      </c>
+      <c r="P11" s="6">
         <v>11845271.89143306</v>
       </c>
-      <c r="Q11">
+      <c r="Q11" s="6">
         <v>0</v>
       </c>
     </row>
@@ -19842,52 +18705,52 @@
       <c r="A12" t="s">
         <v>273</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="6">
         <v>9381.7774113233681</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="5">
         <v>-6.5166760901829237</v>
       </c>
-      <c r="D12">
-        <v>0</v>
-      </c>
-      <c r="E12">
+      <c r="D12" s="5">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5">
         <v>5.0343896711808611</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="6">
         <v>148741.82379735971</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="6">
         <v>74370.911898679857</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="6">
         <v>74370.911898679857</v>
       </c>
-      <c r="I12">
-        <v>0</v>
-      </c>
-      <c r="J12">
-        <v>0</v>
-      </c>
-      <c r="K12">
-        <v>0</v>
-      </c>
-      <c r="L12">
+      <c r="I12" s="6">
+        <v>0</v>
+      </c>
+      <c r="J12" s="6">
+        <v>0</v>
+      </c>
+      <c r="K12" s="6">
+        <v>0</v>
+      </c>
+      <c r="L12" s="6">
         <v>385711.12540703168</v>
       </c>
-      <c r="M12">
+      <c r="M12" s="6">
         <v>710569.37732459186</v>
       </c>
-      <c r="N12">
+      <c r="N12" s="6">
         <v>473600.07571491989</v>
       </c>
-      <c r="O12">
-        <v>0</v>
-      </c>
-      <c r="P12">
+      <c r="O12" s="6">
+        <v>0</v>
+      </c>
+      <c r="P12" s="6">
         <v>300061.24755146692</v>
       </c>
-      <c r="Q12">
+      <c r="Q12" s="6">
         <v>0</v>
       </c>
     </row>
@@ -19895,52 +18758,52 @@
       <c r="A13" t="s">
         <v>274</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="6">
         <v>10875.722527829839</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="5">
         <v>-6.044278189882994</v>
       </c>
-      <c r="D13">
-        <v>0</v>
-      </c>
-      <c r="E13">
+      <c r="D13" s="5">
+        <v>0</v>
+      </c>
+      <c r="E13" s="5">
         <v>4.9847386511287253</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="6">
         <v>12017.673393251969</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="6">
         <v>10005.66472560345</v>
       </c>
-      <c r="H13">
+      <c r="H13" s="6">
         <v>10005.66472560345</v>
       </c>
-      <c r="I13">
-        <v>0</v>
-      </c>
-      <c r="J13">
-        <v>0</v>
-      </c>
-      <c r="K13">
-        <v>0</v>
-      </c>
-      <c r="L13">
+      <c r="I13" s="6">
+        <v>0</v>
+      </c>
+      <c r="J13" s="6">
+        <v>0</v>
+      </c>
+      <c r="K13" s="6">
+        <v>0</v>
+      </c>
+      <c r="L13" s="6">
         <v>282231.50407453772</v>
       </c>
-      <c r="M13">
+      <c r="M13" s="6">
         <v>677567.50018944137</v>
       </c>
-      <c r="N13">
+      <c r="N13" s="6">
         <v>407353.66950815573</v>
       </c>
-      <c r="O13">
-        <v>0</v>
-      </c>
-      <c r="P13">
+      <c r="O13" s="6">
+        <v>0</v>
+      </c>
+      <c r="P13" s="6">
         <v>327467.08392047661</v>
       </c>
-      <c r="Q13">
+      <c r="Q13" s="6">
         <v>0</v>
       </c>
     </row>
@@ -19948,52 +18811,52 @@
       <c r="A14" t="s">
         <v>275</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="6">
         <v>42274.274414881816</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="5">
         <v>-1.2807860584197921</v>
       </c>
-      <c r="D14">
-        <v>0</v>
-      </c>
-      <c r="E14">
+      <c r="D14" s="5">
+        <v>0</v>
+      </c>
+      <c r="E14" s="5">
         <v>2.5860796726634172</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="6">
         <v>549069.84811508202</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="6">
         <v>664478.67296891147</v>
       </c>
-      <c r="H14">
+      <c r="H14" s="6">
         <v>407774.31000719138</v>
       </c>
-      <c r="I14">
-        <v>0</v>
-      </c>
-      <c r="J14">
+      <c r="I14" s="6">
+        <v>0</v>
+      </c>
+      <c r="J14" s="6">
         <v>176991.48534691479</v>
       </c>
-      <c r="K14">
-        <v>0</v>
-      </c>
-      <c r="L14">
+      <c r="K14" s="6">
+        <v>0</v>
+      </c>
+      <c r="L14" s="6">
         <v>831792.08184248838</v>
       </c>
-      <c r="M14">
+      <c r="M14" s="6">
         <v>1016548.172944742</v>
       </c>
-      <c r="N14">
+      <c r="N14" s="6">
         <v>477121.57625561551</v>
       </c>
-      <c r="O14">
-        <v>0</v>
-      </c>
-      <c r="P14">
+      <c r="O14" s="6">
+        <v>0</v>
+      </c>
+      <c r="P14" s="6">
         <v>317012.96233042493</v>
       </c>
-      <c r="Q14">
+      <c r="Q14" s="6">
         <v>0</v>
       </c>
     </row>
@@ -20001,52 +18864,52 @@
       <c r="A15" t="s">
         <v>276</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="6">
         <v>48672</v>
       </c>
-      <c r="C15">
-        <v>0</v>
-      </c>
-      <c r="D15">
-        <v>0</v>
-      </c>
-      <c r="E15">
-        <v>0</v>
-      </c>
-      <c r="F15">
+      <c r="C15" s="5">
+        <v>0</v>
+      </c>
+      <c r="D15" s="5">
+        <v>0</v>
+      </c>
+      <c r="E15" s="5">
+        <v>0</v>
+      </c>
+      <c r="F15" s="6">
         <v>685470.48959999997</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="6">
         <v>685470.48959999997</v>
       </c>
-      <c r="H15">
+      <c r="H15" s="6">
         <v>1370928</v>
       </c>
-      <c r="I15">
-        <v>0</v>
-      </c>
-      <c r="J15">
-        <v>0</v>
-      </c>
-      <c r="K15">
-        <v>0</v>
-      </c>
-      <c r="L15">
+      <c r="I15" s="6">
+        <v>0</v>
+      </c>
+      <c r="J15" s="6">
+        <v>0</v>
+      </c>
+      <c r="K15" s="6">
+        <v>0</v>
+      </c>
+      <c r="L15" s="6">
         <v>685470.48959999997</v>
       </c>
-      <c r="M15">
+      <c r="M15" s="6">
         <v>685470.48959999997</v>
       </c>
-      <c r="N15">
+      <c r="N15" s="6">
         <v>1370928</v>
       </c>
-      <c r="O15">
-        <v>0</v>
-      </c>
-      <c r="P15">
-        <v>0</v>
-      </c>
-      <c r="Q15">
+      <c r="O15" s="6">
+        <v>0</v>
+      </c>
+      <c r="P15" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="6">
         <v>0</v>
       </c>
     </row>
@@ -20054,52 +18917,52 @@
       <c r="A16" t="s">
         <v>277</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="6">
         <v>20555.95319345692</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="5">
         <v>-0.25000150998731557</v>
       </c>
-      <c r="D16">
-        <v>0</v>
-      </c>
-      <c r="E16">
+      <c r="D16" s="5">
+        <v>0</v>
+      </c>
+      <c r="E16" s="5">
         <v>5.839900000000001</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="6">
         <v>1599.22575051335</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="6">
         <v>1175.7890949070379</v>
       </c>
-      <c r="H16">
+      <c r="H16" s="6">
         <v>1175.7890949070379</v>
       </c>
-      <c r="I16">
-        <v>0</v>
-      </c>
-      <c r="J16">
-        <v>0</v>
-      </c>
-      <c r="K16">
-        <v>0</v>
-      </c>
-      <c r="L16">
+      <c r="I16" s="6">
+        <v>0</v>
+      </c>
+      <c r="J16" s="6">
+        <v>0</v>
+      </c>
+      <c r="K16" s="6">
+        <v>0</v>
+      </c>
+      <c r="L16" s="6">
         <v>702648.33383750753</v>
       </c>
-      <c r="M16">
+      <c r="M16" s="6">
         <v>703509.65977615339</v>
       </c>
-      <c r="N16">
+      <c r="N16" s="6">
         <v>2460.5516891592529</v>
       </c>
-      <c r="O16">
-        <v>0</v>
-      </c>
-      <c r="P16">
+      <c r="O16" s="6">
+        <v>0</v>
+      </c>
+      <c r="P16" s="6">
         <v>30011.359029608269</v>
       </c>
-      <c r="Q16">
+      <c r="Q16" s="6">
         <v>0</v>
       </c>
     </row>
@@ -20107,52 +18970,52 @@
       <c r="A17" t="s">
         <v>278</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="6">
         <v>30635</v>
       </c>
-      <c r="C17">
-        <v>0</v>
-      </c>
-      <c r="D17">
+      <c r="C17" s="5">
+        <v>0</v>
+      </c>
+      <c r="D17" s="5">
         <v>-5.0601298473999998</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="5">
         <v>1.8101298474</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="6">
         <v>66918.482616250083</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="6">
         <v>66918.482616250083</v>
       </c>
-      <c r="H17">
+      <c r="H17" s="6">
         <v>66918.482616250083</v>
       </c>
-      <c r="I17">
-        <v>0</v>
-      </c>
-      <c r="J17">
-        <v>0</v>
-      </c>
-      <c r="K17">
-        <v>0</v>
-      </c>
-      <c r="L17">
+      <c r="I17" s="6">
+        <v>0</v>
+      </c>
+      <c r="J17" s="6">
+        <v>0</v>
+      </c>
+      <c r="K17" s="6">
+        <v>0</v>
+      </c>
+      <c r="L17" s="6">
         <v>951702.74915314373</v>
       </c>
-      <c r="M17">
+      <c r="M17" s="6">
         <v>167296.20654062519</v>
       </c>
-      <c r="N17">
+      <c r="N17" s="6">
         <v>851325.0252287687</v>
       </c>
-      <c r="O17">
-        <v>0</v>
-      </c>
-      <c r="P17">
-        <v>0</v>
-      </c>
-      <c r="Q17">
+      <c r="O17" s="6">
+        <v>0</v>
+      </c>
+      <c r="P17" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="6">
         <v>280601.03951844678</v>
       </c>
     </row>
@@ -20160,52 +19023,52 @@
       <c r="A18" t="s">
         <v>279</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="6">
         <v>11983.85</v>
       </c>
-      <c r="C18">
-        <v>0</v>
-      </c>
-      <c r="D18">
+      <c r="C18" s="5">
+        <v>0</v>
+      </c>
+      <c r="D18" s="5">
         <v>5.0601298473999998</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="5">
         <v>1.8101298474</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="6">
         <v>26177.282777892891</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="6">
         <v>26177.282777892891</v>
       </c>
-      <c r="H18">
+      <c r="H18" s="6">
         <v>26177.282777892891</v>
       </c>
-      <c r="I18">
-        <v>0</v>
-      </c>
-      <c r="J18">
-        <v>0</v>
-      </c>
-      <c r="K18">
-        <v>0</v>
-      </c>
-      <c r="L18">
+      <c r="I18" s="6">
+        <v>0</v>
+      </c>
+      <c r="J18" s="6">
+        <v>0</v>
+      </c>
+      <c r="K18" s="6">
+        <v>0</v>
+      </c>
+      <c r="L18" s="6">
         <v>372288.65645304072</v>
       </c>
-      <c r="M18">
+      <c r="M18" s="6">
         <v>65443.206944732206</v>
       </c>
-      <c r="N18">
+      <c r="N18" s="6">
         <v>333022.73228620138</v>
       </c>
-      <c r="O18">
-        <v>0</v>
-      </c>
-      <c r="P18">
-        <v>0</v>
-      </c>
-      <c r="Q18">
+      <c r="O18" s="6">
+        <v>0</v>
+      </c>
+      <c r="P18" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="6">
         <v>-109765.9790250739</v>
       </c>
     </row>
@@ -20213,52 +19076,52 @@
       <c r="A19" t="s">
         <v>280</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="6">
         <v>644813.26594601222</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="5">
         <v>-5.1245107925153039</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="5">
         <v>-0.14636367734288569</v>
       </c>
-      <c r="E19">
+      <c r="E19" s="5">
         <v>4.3141657111563703</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="6">
         <v>9472954.7400160171</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="6">
         <v>10596987.68614725</v>
       </c>
-      <c r="H19">
+      <c r="H19" s="6">
         <v>10521957.30151153</v>
       </c>
-      <c r="I19">
+      <c r="I19" s="6">
         <v>483637.18906450341</v>
       </c>
-      <c r="J19">
+      <c r="J19" s="6">
         <v>2197421.5800634511</v>
       </c>
-      <c r="K19">
+      <c r="K19" s="6">
         <v>-236323.9956939207</v>
       </c>
-      <c r="L19">
+      <c r="L19" s="6">
         <v>21488049.271249719</v>
       </c>
-      <c r="M19">
+      <c r="M19" s="6">
         <v>39531459.073413692</v>
       </c>
-      <c r="N19">
+      <c r="N19" s="6">
         <v>27468960.957587171</v>
       </c>
-      <c r="O19">
-        <v>0</v>
-      </c>
-      <c r="P19">
+      <c r="O19" s="6">
+        <v>0</v>
+      </c>
+      <c r="P19" s="6">
         <v>16452946.00784969</v>
       </c>
-      <c r="Q19">
+      <c r="Q19" s="6">
         <v>170835.0604933729</v>
       </c>
     </row>
@@ -20266,52 +19129,52 @@
       <c r="A20" t="s">
         <v>281</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="6">
         <v>28187.49375044175</v>
       </c>
-      <c r="C20">
-        <v>0</v>
-      </c>
-      <c r="D20">
-        <v>0</v>
-      </c>
-      <c r="E20">
-        <v>0</v>
-      </c>
-      <c r="F20">
-        <v>0</v>
-      </c>
-      <c r="G20">
-        <v>0</v>
-      </c>
-      <c r="H20">
-        <v>0</v>
-      </c>
-      <c r="I20">
-        <v>0</v>
-      </c>
-      <c r="J20">
-        <v>0</v>
-      </c>
-      <c r="K20">
-        <v>0</v>
-      </c>
-      <c r="L20">
-        <v>0</v>
-      </c>
-      <c r="M20">
-        <v>0</v>
-      </c>
-      <c r="N20">
-        <v>0</v>
-      </c>
-      <c r="O20">
-        <v>0</v>
-      </c>
-      <c r="P20">
-        <v>0</v>
-      </c>
-      <c r="Q20">
+      <c r="C20" s="5">
+        <v>0</v>
+      </c>
+      <c r="D20" s="5">
+        <v>0</v>
+      </c>
+      <c r="E20" s="5">
+        <v>0</v>
+      </c>
+      <c r="F20" s="6">
+        <v>0</v>
+      </c>
+      <c r="G20" s="6">
+        <v>0</v>
+      </c>
+      <c r="H20" s="6">
+        <v>0</v>
+      </c>
+      <c r="I20" s="6">
+        <v>0</v>
+      </c>
+      <c r="J20" s="6">
+        <v>0</v>
+      </c>
+      <c r="K20" s="6">
+        <v>0</v>
+      </c>
+      <c r="L20" s="6">
+        <v>0</v>
+      </c>
+      <c r="M20" s="6">
+        <v>0</v>
+      </c>
+      <c r="N20" s="6">
+        <v>0</v>
+      </c>
+      <c r="O20" s="6">
+        <v>0</v>
+      </c>
+      <c r="P20" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="6">
         <v>0</v>
       </c>
     </row>
@@ -20319,52 +19182,52 @@
       <c r="A21" t="s">
         <v>282</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="6">
         <v>673000.75969645393</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="5">
         <v>-4.9098793617822292</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="5">
         <v>-0.14023348331122509</v>
       </c>
-      <c r="E21">
+      <c r="E21" s="5">
         <v>4.1334742078117994</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="6">
         <v>9955109.5568578355</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="6">
         <v>11758101.70950149</v>
       </c>
-      <c r="H21">
+      <c r="H21" s="6">
         <v>11202025.14638547</v>
       </c>
-      <c r="I21">
+      <c r="I21" s="6">
         <v>464229.26849383238</v>
       </c>
-      <c r="J21">
+      <c r="J21" s="6">
         <v>2769482.811175345</v>
       </c>
-      <c r="K21">
+      <c r="K21" s="6">
         <v>-219985.07304531839</v>
       </c>
-      <c r="L21">
+      <c r="L21" s="6">
         <v>21466972.260889929</v>
       </c>
-      <c r="M21">
+      <c r="M21" s="6">
         <v>39480701.906951189</v>
       </c>
-      <c r="N21">
+      <c r="N21" s="6">
         <v>27439232.338249389</v>
       </c>
-      <c r="O21">
+      <c r="O21" s="6">
         <v>848.40165158855962</v>
       </c>
-      <c r="P21">
+      <c r="P21" s="6">
         <v>16427938.81083866</v>
       </c>
-      <c r="Q21">
+      <c r="Q21" s="6">
         <v>170120.81761970819</v>
       </c>
     </row>
@@ -20372,52 +19235,52 @@
       <c r="A22" t="s">
         <v>283</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="6">
         <v>203762.89798054329</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="5">
         <v>-11.420282641214079</v>
       </c>
-      <c r="D22">
-        <v>0</v>
-      </c>
-      <c r="E22">
+      <c r="D22" s="5">
+        <v>0</v>
+      </c>
+      <c r="E22" s="5">
         <v>5.5497794877707518</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="6">
         <v>348952878.90076488</v>
       </c>
-      <c r="G22">
+      <c r="G22" s="6">
         <v>174476439.45038241</v>
       </c>
-      <c r="H22">
+      <c r="H22" s="6">
         <v>174476439.45038241</v>
       </c>
-      <c r="I22">
-        <v>0</v>
-      </c>
-      <c r="J22">
-        <v>0</v>
-      </c>
-      <c r="K22">
-        <v>0</v>
-      </c>
-      <c r="L22">
+      <c r="I22" s="6">
+        <v>0</v>
+      </c>
+      <c r="J22" s="6">
+        <v>0</v>
+      </c>
+      <c r="K22" s="6">
+        <v>0</v>
+      </c>
+      <c r="L22" s="6">
         <v>353322422.41947103</v>
       </c>
-      <c r="M22">
+      <c r="M22" s="6">
         <v>207327686.3988122</v>
       </c>
-      <c r="N22">
+      <c r="N22" s="6">
         <v>202958142.88010591</v>
       </c>
-      <c r="O22">
-        <v>0</v>
-      </c>
-      <c r="P22">
+      <c r="O22" s="6">
+        <v>0</v>
+      </c>
+      <c r="P22" s="6">
         <v>-5223343.0341883227</v>
       </c>
-      <c r="Q22">
+      <c r="Q22" s="6">
         <v>0</v>
       </c>
     </row>
@@ -20425,52 +19288,52 @@
       <c r="A23" t="s">
         <v>284</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="6">
         <v>69006.036596403326</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="5">
         <v>-11.420282641214079</v>
       </c>
-      <c r="D23">
-        <v>0</v>
-      </c>
-      <c r="E23">
+      <c r="D23" s="5">
+        <v>0</v>
+      </c>
+      <c r="E23" s="5">
         <v>5.5497794877707518</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="6">
         <v>967788.48302954319</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="6">
         <v>617257.07610674994</v>
       </c>
-      <c r="H23">
+      <c r="H23" s="6">
         <v>617257.07610674994</v>
       </c>
-      <c r="I23">
-        <v>0</v>
-      </c>
-      <c r="J23">
-        <v>0</v>
-      </c>
-      <c r="K23">
-        <v>0</v>
-      </c>
-      <c r="L23">
+      <c r="I23" s="6">
+        <v>0</v>
+      </c>
+      <c r="J23" s="6">
+        <v>0</v>
+      </c>
+      <c r="K23" s="6">
+        <v>0</v>
+      </c>
+      <c r="L23" s="6">
         <v>3089348.0474239378</v>
       </c>
-      <c r="M23">
+      <c r="M23" s="6">
         <v>11742610.963531779</v>
       </c>
-      <c r="N23">
+      <c r="N23" s="6">
         <v>9621051.3991373889</v>
       </c>
-      <c r="O23">
-        <v>0</v>
-      </c>
-      <c r="P23">
+      <c r="O23" s="6">
+        <v>0</v>
+      </c>
+      <c r="P23" s="6">
         <v>4337166.2849609861</v>
       </c>
-      <c r="Q23">
+      <c r="Q23" s="6">
         <v>0</v>
       </c>
     </row>
@@ -20478,52 +19341,52 @@
       <c r="A24" t="s">
         <v>285</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="6">
         <v>945769.69427340059</v>
       </c>
-      <c r="C24">
+      <c r="C24" s="5">
         <v>-7.3209600058004138</v>
       </c>
-      <c r="D24">
+      <c r="D24" s="5">
         <v>-9.9788818963839829E-2</v>
       </c>
-      <c r="E24">
+      <c r="E24" s="5">
         <v>4.5980146245874653</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="6">
         <v>499865525.61414582</v>
       </c>
-      <c r="G24">
+      <c r="G24" s="6">
         <v>342629218.42514449</v>
       </c>
-      <c r="H24">
+      <c r="H24" s="6">
         <v>343480100.46718019</v>
       </c>
-      <c r="I24">
+      <c r="I24" s="6">
         <v>691780.40703059547</v>
       </c>
-      <c r="J24">
+      <c r="J24" s="6">
         <v>-12757977.77672961</v>
       </c>
-      <c r="K24">
+      <c r="K24" s="6">
         <v>-263827.11582223681</v>
       </c>
-      <c r="L24">
+      <c r="L24" s="6">
         <v>378481085.78667837</v>
       </c>
-      <c r="M24">
+      <c r="M24" s="6">
         <v>271925264.04825127</v>
       </c>
-      <c r="N24">
+      <c r="N24" s="6">
         <v>252790348.33755529</v>
       </c>
-      <c r="O24">
+      <c r="O24" s="6">
         <v>848.40165158855962</v>
       </c>
-      <c r="P24">
+      <c r="P24" s="6">
         <v>19078409.288633171</v>
       </c>
-      <c r="Q24">
+      <c r="Q24" s="6">
         <v>170120.81761970819</v>
       </c>
     </row>

</xml_diff>